<commit_message>
Curtin: show unit codes for specialisation-titled rows
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01EZa6h9SpqLeB7ZbHz6KiwN
</commit_message>
<xml_diff>
--- a/curriculum_mapping_2026-27/CurriculumMapping_Geo_1_ReviewEntry_OK.xlsx
+++ b/curriculum_mapping_2026-27/CurriculumMapping_Geo_1_ReviewEntry_OK.xlsx
@@ -4686,214 +4686,214 @@
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="7" t="inlineStr">
+      <c r="A21" s="3" t="inlineStr">
         <is>
           <t>Curtin University — Australia</t>
         </is>
       </c>
-      <c r="B21" s="7" t="inlineStr">
+      <c r="B21" s="3" t="inlineStr">
         <is>
           <t>Geography BA</t>
         </is>
       </c>
-      <c r="C21" s="7" t="inlineStr">
+      <c r="C21" s="3" t="inlineStr">
+        <is>
+          <t>SOES270 RETHINKING NATURE: ENVIRONMENTAL KNOWLEDGE, SCIENCE AND SOCIETY</t>
+        </is>
+      </c>
+      <c r="D21" s="3" t="inlineStr">
+        <is>
+          <t>Level 5</t>
+        </is>
+      </c>
+      <c r="E21" s="3" t="inlineStr">
+        <is>
+          <t>GEOG1000 Human Geography (25 credits)</t>
+        </is>
+      </c>
+      <c r="F21" s="3" t="inlineStr">
+        <is>
+          <t>Undergraduate</t>
+        </is>
+      </c>
+      <c r="G21" s="3" t="inlineStr">
+        <is>
+          <t>Optional</t>
+        </is>
+      </c>
+      <c r="H21" s="3" t="inlineStr">
+        <is>
+          <t>Semester 1 2026 (2027 not yet listed) - unit GEOG1000</t>
+        </is>
+      </c>
+      <c r="I21" s="3" t="n"/>
+      <c r="J21" s="3" t="inlineStr">
+        <is>
+          <t>Host: https://www.curtin.edu.au/study/offering/course-ug-geography-specialisation--spuc-geogr/ | UoL: https://www.liverpool.ac.uk/courses/geography-ba-hons</t>
+        </is>
+      </c>
+      <c r="K21" s="3" t="inlineStr">
+        <is>
+          <t>Original row; TERM LIKELY (2026/27 timetable not yet published or pattern only): Semester 1 2026 (2027 not yet listed) - unit GEOG1000 [https://handbook.curtin.edu.au/]</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="3" t="inlineStr">
+        <is>
+          <t>Curtin University — Australia</t>
+        </is>
+      </c>
+      <c r="B22" s="3" t="inlineStr">
+        <is>
+          <t>Geography BA</t>
+        </is>
+      </c>
+      <c r="C22" s="3" t="inlineStr">
+        <is>
+          <t>SOES224 POLITICAL ECONOMIES OF CRISIS AND CHANGE</t>
+        </is>
+      </c>
+      <c r="D22" s="3" t="inlineStr">
+        <is>
+          <t>Level 5</t>
+        </is>
+      </c>
+      <c r="E22" s="3" t="inlineStr">
+        <is>
+          <t>GEOG2001 Geographies of Food Security (25 credits)</t>
+        </is>
+      </c>
+      <c r="F22" s="3" t="inlineStr">
+        <is>
+          <t>Undergraduate</t>
+        </is>
+      </c>
+      <c r="G22" s="3" t="inlineStr">
+        <is>
+          <t>Optional</t>
+        </is>
+      </c>
+      <c r="H22" s="3" t="inlineStr">
+        <is>
+          <t>Semester 1 2027 (Curtin Perth) - unit GEOG2001</t>
+        </is>
+      </c>
+      <c r="I22" s="3" t="n"/>
+      <c r="J22" s="3" t="inlineStr">
+        <is>
+          <t>Host: https://www.curtin.edu.au/study/offering/course-ug-geography-specialisation--spuc-geogr/ | UoL: https://www.liverpool.ac.uk/courses/geography-ba-hons</t>
+        </is>
+      </c>
+      <c r="K22" s="3" t="inlineStr">
+        <is>
+          <t>Original row; TERM VERIFIED Oct 2026: Semester 1 2027 (Curtin Perth) - unit GEOG2001 [https://handbook.curtin.edu.au/]</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="7" t="inlineStr">
+        <is>
+          <t>Curtin University — Australia</t>
+        </is>
+      </c>
+      <c r="B23" s="7" t="inlineStr">
+        <is>
+          <t>Geography BA</t>
+        </is>
+      </c>
+      <c r="C23" s="7" t="inlineStr">
         <is>
           <t>SOES276 BA GEOGRAPHY EUROPEAN FIELD CLASS</t>
         </is>
       </c>
-      <c r="D21" s="7" t="inlineStr">
-        <is>
-          <t>Level 5</t>
-        </is>
-      </c>
-      <c r="E21" s="7" t="inlineStr">
+      <c r="D23" s="7" t="inlineStr">
+        <is>
+          <t>Level 5</t>
+        </is>
+      </c>
+      <c r="E23" s="7" t="inlineStr">
         <is>
           <t>GEOG2002 Fieldwork Skills (25 credits)</t>
         </is>
       </c>
-      <c r="F21" s="7" t="inlineStr">
+      <c r="F23" s="7" t="inlineStr">
         <is>
           <t>Level 2</t>
         </is>
       </c>
-      <c r="G21" s="7" t="inlineStr">
-        <is>
-          <t>Optional</t>
-        </is>
-      </c>
-      <c r="H21" s="7" t="inlineStr">
+      <c r="G23" s="7" t="inlineStr">
+        <is>
+          <t>Optional</t>
+        </is>
+      </c>
+      <c r="H23" s="7" t="inlineStr">
         <is>
           <t>2026 Semester 1 (Curtin Perth); 2027 Semester 1 (Curtin Perth)</t>
         </is>
       </c>
-      <c r="I21" s="7" t="n"/>
-      <c r="J21" s="7" t="inlineStr">
+      <c r="I23" s="7" t="n"/>
+      <c r="J23" s="7" t="inlineStr">
         <is>
           <t>Host: https://handbook.curtin.edu.au/units/unit-ug-fieldwork-skills--geog2002v1 | NEW (Jul 2025 handbook, not previously in this file) - verified in current host catalogue, Oct 2026 | UoL match is a SUGGESTION for department review (programme LOs, not close module match)</t>
         </is>
       </c>
-      <c r="K21" s="7" t="inlineStr">
+      <c r="K23" s="7" t="inlineStr">
         <is>
           <t>Added Oct 2026: July 2025 handbook module verified in current catalogue; UoL match is a suggestion for review</t>
         </is>
       </c>
     </row>
-    <row r="22">
-      <c r="A22" s="7" t="inlineStr">
+    <row r="24">
+      <c r="A24" s="7" t="inlineStr">
         <is>
           <t>Curtin University — Australia</t>
         </is>
       </c>
-      <c r="B22" s="7" t="inlineStr">
+      <c r="B24" s="7" t="inlineStr">
         <is>
           <t>Geography BA</t>
         </is>
       </c>
-      <c r="C22" s="7" t="inlineStr">
+      <c r="C24" s="7" t="inlineStr">
         <is>
           <t>SOES270 RETHINKING NATURE: ENVIRONMENTAL KNOWLEDGE, SCIENCE AND SOCIETY</t>
         </is>
       </c>
-      <c r="D22" s="7" t="inlineStr">
-        <is>
-          <t>Level 5</t>
-        </is>
-      </c>
-      <c r="E22" s="7" t="inlineStr">
+      <c r="D24" s="7" t="inlineStr">
+        <is>
+          <t>Level 5</t>
+        </is>
+      </c>
+      <c r="E24" s="7" t="inlineStr">
         <is>
           <t>GEOG3001 Sustainable Livelihoods (25 credits)</t>
         </is>
       </c>
-      <c r="F22" s="7" t="inlineStr">
+      <c r="F24" s="7" t="inlineStr">
         <is>
           <t>Level 3</t>
         </is>
       </c>
-      <c r="G22" s="7" t="inlineStr">
-        <is>
-          <t>Optional</t>
-        </is>
-      </c>
-      <c r="H22" s="7" t="inlineStr">
+      <c r="G24" s="7" t="inlineStr">
+        <is>
+          <t>Optional</t>
+        </is>
+      </c>
+      <c r="H24" s="7" t="inlineStr">
         <is>
           <t>2026 Semester 1 (Curtin Perth); 2027 Semester 1 (Curtin Perth)</t>
         </is>
       </c>
-      <c r="I22" s="7" t="n"/>
-      <c r="J22" s="7" t="inlineStr">
+      <c r="I24" s="7" t="n"/>
+      <c r="J24" s="7" t="inlineStr">
         <is>
           <t>Host: https://handbook.curtin.edu.au/units/unit-ug-sustainable-livelihoods--geog3001v1 | NEW (Jul 2025 handbook, not previously in this file) - verified in current host catalogue, Oct 2026 | UoL match is a SUGGESTION for department review (programme LOs, not close module match)</t>
         </is>
       </c>
-      <c r="K22" s="7" t="inlineStr">
+      <c r="K24" s="7" t="inlineStr">
         <is>
           <t>Added Oct 2026: July 2025 handbook module verified in current catalogue; UoL match is a suggestion for review</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" s="3" t="inlineStr">
-        <is>
-          <t>Curtin University — Australia</t>
-        </is>
-      </c>
-      <c r="B23" s="3" t="inlineStr">
-        <is>
-          <t>Geography BA</t>
-        </is>
-      </c>
-      <c r="C23" s="3" t="inlineStr">
-        <is>
-          <t>SOES224 POLITICAL ECONOMIES OF CRISIS AND CHANGE</t>
-        </is>
-      </c>
-      <c r="D23" s="3" t="inlineStr">
-        <is>
-          <t>Level 5</t>
-        </is>
-      </c>
-      <c r="E23" s="3" t="inlineStr">
-        <is>
-          <t>Geographies of Food Security [current specialisation title; unit code not exposed on public page]</t>
-        </is>
-      </c>
-      <c r="F23" s="3" t="inlineStr">
-        <is>
-          <t>Undergraduate</t>
-        </is>
-      </c>
-      <c r="G23" s="3" t="inlineStr">
-        <is>
-          <t>Optional</t>
-        </is>
-      </c>
-      <c r="H23" s="3" t="inlineStr">
-        <is>
-          <t>Semester 1 2027 (Curtin Perth) - unit GEOG2001</t>
-        </is>
-      </c>
-      <c r="I23" s="3" t="n"/>
-      <c r="J23" s="3" t="inlineStr">
-        <is>
-          <t>Host: https://www.curtin.edu.au/study/offering/course-ug-geography-specialisation--spuc-geogr/ | UoL: https://www.liverpool.ac.uk/courses/geography-ba-hons</t>
-        </is>
-      </c>
-      <c r="K23" s="3" t="inlineStr">
-        <is>
-          <t>Original row; TERM VERIFIED Oct 2026: Semester 1 2027 (Curtin Perth) - unit GEOG2001 [https://handbook.curtin.edu.au/]</t>
-        </is>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" s="3" t="inlineStr">
-        <is>
-          <t>Curtin University — Australia</t>
-        </is>
-      </c>
-      <c r="B24" s="3" t="inlineStr">
-        <is>
-          <t>Geography BA</t>
-        </is>
-      </c>
-      <c r="C24" s="3" t="inlineStr">
-        <is>
-          <t>SOES270 RETHINKING NATURE: ENVIRONMENTAL KNOWLEDGE, SCIENCE AND SOCIETY</t>
-        </is>
-      </c>
-      <c r="D24" s="3" t="inlineStr">
-        <is>
-          <t>Level 5</t>
-        </is>
-      </c>
-      <c r="E24" s="3" t="inlineStr">
-        <is>
-          <t>Human Geography [current specialisation title; unit code not exposed on public page]</t>
-        </is>
-      </c>
-      <c r="F24" s="3" t="inlineStr">
-        <is>
-          <t>Undergraduate</t>
-        </is>
-      </c>
-      <c r="G24" s="3" t="inlineStr">
-        <is>
-          <t>Optional</t>
-        </is>
-      </c>
-      <c r="H24" s="3" t="inlineStr">
-        <is>
-          <t>Semester 1 2026 (2027 not yet listed) - unit GEOG1000</t>
-        </is>
-      </c>
-      <c r="I24" s="3" t="n"/>
-      <c r="J24" s="3" t="inlineStr">
-        <is>
-          <t>Host: https://www.curtin.edu.au/study/offering/course-ug-geography-specialisation--spuc-geogr/ | UoL: https://www.liverpool.ac.uk/courses/geography-ba-hons</t>
-        </is>
-      </c>
-      <c r="K24" s="3" t="inlineStr">
-        <is>
-          <t>Original row; TERM LIKELY (2026/27 timetable not yet published or pattern only): Semester 1 2026 (2027 not yet listed) - unit GEOG1000 [https://handbook.curtin.edu.au/]</t>
         </is>
       </c>
     </row>
@@ -32862,7 +32862,7 @@
       </c>
       <c r="E28" s="9" t="inlineStr">
         <is>
-          <t>Adaptation to Hazards [current specialisation title; unit code not exposed on public page]</t>
+          <t>Adaptation to Hazards (specialisation title, not a Curtin unit)</t>
         </is>
       </c>
       <c r="F28" s="9" t="inlineStr">

</xml_diff>

<commit_message>
UTD GEOS Fall 2026 checked
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01EZa6h9SpqLeB7ZbHz6KiwN
</commit_message>
<xml_diff>
--- a/curriculum_mapping_2026-27/CurriculumMapping_Geo_1_ReviewEntry_OK.xlsx
+++ b/curriculum_mapping_2026-27/CurriculumMapping_Geo_1_ReviewEntry_OK.xlsx
@@ -15,7 +15,7 @@
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Geography BA'!$A$1:$K$264</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Geography BSc'!$A$1:$K$261</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Rows removed (not usable)'!$A$1:$K$251</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Rows removed (not usable)'!$A$1:$K$252</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -2767,17 +2767,17 @@
         </is>
       </c>
       <c r="C64" s="3" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="D64" s="3" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="E64" s="3" t="n">
         <v>4</v>
       </c>
-      <c r="F64" s="4" t="inlineStr">
-        <is>
-          <t>Meets minimum, little choice: 5 modules with confirmed 2026/27 term, 4 needed (+2 more with unverified term)</t>
+      <c r="F64" s="3" t="inlineStr">
+        <is>
+          <t>OK: 7 modules with confirmed 2026/27 term, 4 needed</t>
         </is>
       </c>
       <c r="G64" s="3" t="inlineStr">
@@ -2789,7 +2789,7 @@
         <v>7</v>
       </c>
       <c r="I64" s="3" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="65">
@@ -27390,108 +27390,108 @@
       </c>
     </row>
     <row r="184">
-      <c r="A184" s="4" t="inlineStr">
+      <c r="A184" s="3" t="inlineStr">
         <is>
           <t>University of Texas at Dallas — USA</t>
         </is>
       </c>
-      <c r="B184" s="4" t="inlineStr">
+      <c r="B184" s="3" t="inlineStr">
         <is>
           <t>Geography BSc</t>
         </is>
       </c>
-      <c r="C184" s="4" t="inlineStr">
+      <c r="C184" s="3" t="inlineStr">
         <is>
           <t>SOES214 CHANGING ENVIRONMENTS</t>
         </is>
       </c>
-      <c r="D184" s="4" t="inlineStr">
-        <is>
-          <t>Level 5</t>
-        </is>
-      </c>
-      <c r="E184" s="4" t="inlineStr">
+      <c r="D184" s="3" t="inlineStr">
+        <is>
+          <t>Level 5</t>
+        </is>
+      </c>
+      <c r="E184" s="3" t="inlineStr">
         <is>
           <t>GEOS2310 Environmental Geosciences (3)</t>
         </is>
       </c>
-      <c r="F184" s="4" t="inlineStr">
+      <c r="F184" s="3" t="inlineStr">
         <is>
           <t>Level 2</t>
         </is>
       </c>
-      <c r="G184" s="4" t="inlineStr">
-        <is>
-          <t>Optional</t>
-        </is>
-      </c>
-      <c r="H184" s="4" t="inlineStr">
-        <is>
-          <t>2026/27 catalogue verified; exact semester not specified</t>
-        </is>
-      </c>
-      <c r="I184" s="4" t="n"/>
-      <c r="J184" s="4" t="inlineStr">
+      <c r="G184" s="3" t="inlineStr">
+        <is>
+          <t>Optional</t>
+        </is>
+      </c>
+      <c r="H184" s="3" t="inlineStr">
+        <is>
+          <t>Fall 2026 (section .0w1, online)</t>
+        </is>
+      </c>
+      <c r="I184" s="3" t="n"/>
+      <c r="J184" s="3" t="inlineStr">
         <is>
           <t>Host: https://catalog.utdallas.edu/2026/undergraduate/courses/geog | UoL: https://www.liverpool.ac.uk/courses/geography-bsc-hons</t>
         </is>
       </c>
-      <c r="K184" s="4" t="inlineStr">
-        <is>
-          <t>Original row; TERM NOT VERIFIED: Catalogue frequency code Y: offered once a year (term not stated) (CourseBook is bot-protected; Fall 2026 section not checked) [https://catalog.utdallas.edu/now/undergraduate/courses/geos2310]</t>
+      <c r="K184" s="3" t="inlineStr">
+        <is>
+          <t>Original row; TERM VERIFIED Oct 2026: Fall 2026 (section .0w1, online) — Online section only [https://coursebook.utdallas.edu/search/geos/term_26f (UTD CourseBook 26F/26S - checked manually Oct 2026)]</t>
         </is>
       </c>
     </row>
     <row r="185">
-      <c r="A185" s="4" t="inlineStr">
+      <c r="A185" s="8" t="inlineStr">
         <is>
           <t>University of Texas at Dallas — USA</t>
         </is>
       </c>
-      <c r="B185" s="4" t="inlineStr">
+      <c r="B185" s="8" t="inlineStr">
         <is>
           <t>Geography BSc</t>
         </is>
       </c>
-      <c r="C185" s="4" t="inlineStr">
-        <is>
-          <t>SOES270 RETHINKING NATURE: ENVIRONMENTAL KNOWLEDGE, SCIENCE AND SOCIETY</t>
-        </is>
-      </c>
-      <c r="D185" s="4" t="inlineStr">
-        <is>
-          <t>Level 5</t>
-        </is>
-      </c>
-      <c r="E185" s="4" t="inlineStr">
-        <is>
-          <t>GEOS2312 Soils in a Sustainable Environment (3)</t>
-        </is>
-      </c>
-      <c r="F185" s="4" t="inlineStr">
-        <is>
-          <t>Level 2</t>
-        </is>
-      </c>
-      <c r="G185" s="4" t="inlineStr">
-        <is>
-          <t>Optional</t>
-        </is>
-      </c>
-      <c r="H185" s="4" t="inlineStr">
-        <is>
-          <t>2026/27 catalogue verified; exact semester not specified</t>
-        </is>
-      </c>
-      <c r="I185" s="4" t="n"/>
-      <c r="J185" s="4" t="inlineStr">
-        <is>
-          <t>Host: https://catalog.utdallas.edu/2026/undergraduate/courses/geog | UoL: https://www.liverpool.ac.uk/courses/geography-bsc-hons</t>
-        </is>
-      </c>
-      <c r="K185" s="4" t="inlineStr">
-        <is>
-          <t>Original row; TERM NOT VERIFIED: Catalogue frequency code Y: offered once a year (term not stated) (CourseBook is bot-protected; Fall 2026 section not checked) [https://catalog.utdallas.edu/now/undergraduate/courses/geos2312]</t>
+      <c r="C185" s="8" t="inlineStr">
+        <is>
+          <t>SOES280 HYDROCLIMATE</t>
+        </is>
+      </c>
+      <c r="D185" s="8" t="inlineStr">
+        <is>
+          <t>Level 5</t>
+        </is>
+      </c>
+      <c r="E185" s="8" t="inlineStr">
+        <is>
+          <t>GEOS4430 Hydrogeology and Aqueous Geochemistry (4)</t>
+        </is>
+      </c>
+      <c r="F185" s="8" t="inlineStr">
+        <is>
+          <t>Level 4</t>
+        </is>
+      </c>
+      <c r="G185" s="8" t="inlineStr">
+        <is>
+          <t>Optional</t>
+        </is>
+      </c>
+      <c r="H185" s="8" t="inlineStr">
+        <is>
+          <t>Fall 2026 - UTD CourseBook (26F), checked manually Oct 2026</t>
+        </is>
+      </c>
+      <c r="I185" s="8" t="n"/>
+      <c r="J185" s="8" t="inlineStr">
+        <is>
+          <t>Host: https://coursebook.utdallas.edu/search/geos/term_26f (UTD CourseBook 26F/26S - checked manually Oct 2026) | NEW (Oct 2026 deep check: module confirmed in the 2026/27 timetable for the exchange period) | UoL match is a SUGGESTION for department review</t>
+        </is>
+      </c>
+      <c r="K185" s="8" t="inlineStr">
+        <is>
+          <t>Added Oct 2026 (deep check): verified in 2026/27 timetable; UoL match is a suggestion for review</t>
         </is>
       </c>
     </row>
@@ -31535,7 +31535,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K251"/>
+  <dimension ref="A1:K252"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -39889,7 +39889,7 @@
       </c>
       <c r="C158" s="10" t="inlineStr">
         <is>
-          <t>SOES269 GIS FOR THE NATURAL ENVIRONMENT</t>
+          <t>SOES270 RETHINKING NATURE: ENVIRONMENTAL KNOWLEDGE, SCIENCE AND SOCIETY</t>
         </is>
       </c>
       <c r="D158" s="10" t="inlineStr">
@@ -39899,12 +39899,12 @@
       </c>
       <c r="E158" s="10" t="inlineStr">
         <is>
-          <t>GISC2309 Principles of Geospatial Information Sciences (3)</t>
+          <t>GEOS2312 Soils in a Sustainable Environment (3)</t>
         </is>
       </c>
       <c r="F158" s="10" t="inlineStr">
         <is>
-          <t>Level 3</t>
+          <t>Level 2</t>
         </is>
       </c>
       <c r="G158" s="10" t="inlineStr">
@@ -39914,7 +39914,7 @@
       </c>
       <c r="H158" s="10" t="inlineStr">
         <is>
-          <t>Spring 2027</t>
+          <t>2026/27 catalogue verified; exact semester not specified</t>
         </is>
       </c>
       <c r="I158" s="10" t="n"/>
@@ -39925,7 +39925,7 @@
       </c>
       <c r="K158" s="10" t="inlineStr">
         <is>
-          <t>Original row; Wrong term for partner semester (Fall Semester [Sep-Dec))</t>
+          <t>Original row; NOT OFFERED 2026/27: Not in Fall 2026 or Spring 2026 CourseBook [https://coursebook.utdallas.edu/search/geos/term_26f (UTD CourseBook 26F/26S - checked manually Oct 2026)]</t>
         </is>
       </c>
     </row>
@@ -39952,7 +39952,7 @@
       </c>
       <c r="E159" s="10" t="inlineStr">
         <is>
-          <t>GISC4325 Introduction to Remote Sensing (3)</t>
+          <t>GISC2309 Principles of Geospatial Information Sciences (3)</t>
         </is>
       </c>
       <c r="F159" s="10" t="inlineStr">
@@ -40005,7 +40005,7 @@
       </c>
       <c r="E160" s="10" t="inlineStr">
         <is>
-          <t>GISC4382 GIS Database and Modeling (3)</t>
+          <t>GISC4325 Introduction to Remote Sensing (3)</t>
         </is>
       </c>
       <c r="F160" s="10" t="inlineStr">
@@ -40038,17 +40038,17 @@
     <row r="161">
       <c r="A161" s="10" t="inlineStr">
         <is>
-          <t>University of Toronto - Mississauga Campus — Canada</t>
+          <t>University of Texas at Dallas — USA</t>
         </is>
       </c>
       <c r="B161" s="10" t="inlineStr">
         <is>
-          <t>Geography BA</t>
+          <t>Geography BSc</t>
         </is>
       </c>
       <c r="C161" s="10" t="inlineStr">
         <is>
-          <t>SOES270 RETHINKING NATURE: ENVIRONMENTAL KNOWLEDGE, SCIENCE AND SOCIETY</t>
+          <t>SOES269 GIS FOR THE NATURAL ENVIRONMENT</t>
         </is>
       </c>
       <c r="D161" s="10" t="inlineStr">
@@ -40058,12 +40058,12 @@
       </c>
       <c r="E161" s="10" t="inlineStr">
         <is>
-          <t>GGR111H5 Human Geography</t>
+          <t>GISC4382 GIS Database and Modeling (3)</t>
         </is>
       </c>
       <c r="F161" s="10" t="inlineStr">
         <is>
-          <t>Level 1</t>
+          <t>Level 3</t>
         </is>
       </c>
       <c r="G161" s="10" t="inlineStr">
@@ -40073,18 +40073,18 @@
       </c>
       <c r="H161" s="10" t="inlineStr">
         <is>
-          <t>2026/27 course verified; Fall/Winter offering not confirmed on public timetable</t>
+          <t>Spring 2027</t>
         </is>
       </c>
       <c r="I161" s="10" t="n"/>
       <c r="J161" s="10" t="inlineStr">
         <is>
-          <t>Host: https://www.utm.utoronto.ca/geography/undergraduate/courses/physical-geography-course-list | UoL: https://www.liverpool.ac.uk/courses/geography-ba-hons</t>
+          <t>Host: https://catalog.utdallas.edu/2026/undergraduate/courses/geog | UoL: https://www.liverpool.ac.uk/courses/geography-bsc-hons</t>
         </is>
       </c>
       <c r="K161" s="10" t="inlineStr">
         <is>
-          <t>Original row; WRONG TERM 2026/27: Winter 2027 (S) only [https://ttb.utoronto.ca/]</t>
+          <t>Original row; Wrong term for partner semester (Fall Semester [Sep-Dec))</t>
         </is>
       </c>
     </row>
@@ -40101,7 +40101,7 @@
       </c>
       <c r="C162" s="10" t="inlineStr">
         <is>
-          <t>SOES275 SOCIAL AND CULTURAL GEOGRAPHIES</t>
+          <t>SOES270 RETHINKING NATURE: ENVIRONMENTAL KNOWLEDGE, SCIENCE AND SOCIETY</t>
         </is>
       </c>
       <c r="D162" s="10" t="inlineStr">
@@ -40111,12 +40111,12 @@
       </c>
       <c r="E162" s="10" t="inlineStr">
         <is>
-          <t>GGR208H5 Population Geography</t>
+          <t>GGR111H5 Human Geography</t>
         </is>
       </c>
       <c r="F162" s="10" t="inlineStr">
         <is>
-          <t>Level 2</t>
+          <t>Level 1</t>
         </is>
       </c>
       <c r="G162" s="10" t="inlineStr">
@@ -40154,7 +40154,7 @@
       </c>
       <c r="C163" s="10" t="inlineStr">
         <is>
-          <t>SOES270 RETHINKING NATURE: ENVIRONMENTAL KNOWLEDGE, SCIENCE AND SOCIETY</t>
+          <t>SOES275 SOCIAL AND CULTURAL GEOGRAPHIES</t>
         </is>
       </c>
       <c r="D163" s="10" t="inlineStr">
@@ -40164,12 +40164,12 @@
       </c>
       <c r="E163" s="10" t="inlineStr">
         <is>
-          <t>GGR307H5 Environmental Soil Science (0.5 credit (half course))</t>
+          <t>GGR208H5 Population Geography</t>
         </is>
       </c>
       <c r="F163" s="10" t="inlineStr">
         <is>
-          <t>Level 3</t>
+          <t>Level 2</t>
         </is>
       </c>
       <c r="G163" s="10" t="inlineStr">
@@ -40179,18 +40179,18 @@
       </c>
       <c r="H163" s="10" t="inlineStr">
         <is>
-          <t>Fall/Winter: check timetable</t>
+          <t>2026/27 course verified; Fall/Winter offering not confirmed on public timetable</t>
         </is>
       </c>
       <c r="I163" s="10" t="n"/>
       <c r="J163" s="10" t="inlineStr">
         <is>
-          <t>Host: https://utm.calendar.utoronto.ca/course/ggr307h5 | NEW (Jul 2025 handbook, not previously in this file) - verified in current host catalogue, Oct 2026 | UoL match is a SUGGESTION for department review (programme LOs, not close module match)</t>
+          <t>Host: https://www.utm.utoronto.ca/geography/undergraduate/courses/physical-geography-course-list | UoL: https://www.liverpool.ac.uk/courses/geography-ba-hons</t>
         </is>
       </c>
       <c r="K163" s="10" t="inlineStr">
         <is>
-          <t>Added Oct 2026: July 2025 handbook module verified in current catalogue; UoL match is a suggestion for review; NOT OFFERED 2026/27: Not in the 2026-27 timetable (no Fall 2026 or Winter 2027 section) [https://ttb.utoronto.ca/]</t>
+          <t>Original row; WRONG TERM 2026/27: Winter 2027 (S) only [https://ttb.utoronto.ca/]</t>
         </is>
       </c>
     </row>
@@ -40217,7 +40217,7 @@
       </c>
       <c r="E164" s="10" t="inlineStr">
         <is>
-          <t>GGR387H5 Food and Globalization (0.5 credit (half course))</t>
+          <t>GGR307H5 Environmental Soil Science (0.5 credit (half course))</t>
         </is>
       </c>
       <c r="F164" s="10" t="inlineStr">
@@ -40238,7 +40238,7 @@
       <c r="I164" s="10" t="n"/>
       <c r="J164" s="10" t="inlineStr">
         <is>
-          <t>Host: https://utm.calendar.utoronto.ca/course/ggr387h5 | NEW (Jul 2025 handbook, not previously in this file) - verified in current host catalogue, Oct 2026 | UoL match is a SUGGESTION for department review (programme LOs, not close module match)</t>
+          <t>Host: https://utm.calendar.utoronto.ca/course/ggr307h5 | NEW (Jul 2025 handbook, not previously in this file) - verified in current host catalogue, Oct 2026 | UoL match is a SUGGESTION for department review (programme LOs, not close module match)</t>
         </is>
       </c>
       <c r="K164" s="10" t="inlineStr">
@@ -40255,12 +40255,12 @@
       </c>
       <c r="B165" s="10" t="inlineStr">
         <is>
-          <t>Geography BSc</t>
+          <t>Geography BA</t>
         </is>
       </c>
       <c r="C165" s="10" t="inlineStr">
         <is>
-          <t>SOES218 GEOMORPHOLOGY: PROCESSES AND FORMS</t>
+          <t>SOES270 RETHINKING NATURE: ENVIRONMENTAL KNOWLEDGE, SCIENCE AND SOCIETY</t>
         </is>
       </c>
       <c r="D165" s="10" t="inlineStr">
@@ -40270,12 +40270,12 @@
       </c>
       <c r="E165" s="10" t="inlineStr">
         <is>
-          <t>GGR201H5 Introduction to Geomorphology</t>
+          <t>GGR387H5 Food and Globalization (0.5 credit (half course))</t>
         </is>
       </c>
       <c r="F165" s="10" t="inlineStr">
         <is>
-          <t>Level 2</t>
+          <t>Level 3</t>
         </is>
       </c>
       <c r="G165" s="10" t="inlineStr">
@@ -40285,18 +40285,18 @@
       </c>
       <c r="H165" s="10" t="inlineStr">
         <is>
-          <t>Winter 2027</t>
+          <t>Fall/Winter: check timetable</t>
         </is>
       </c>
       <c r="I165" s="10" t="n"/>
       <c r="J165" s="10" t="inlineStr">
         <is>
-          <t>Host: https://www.utm.utoronto.ca/geography/undergraduate/courses/physical-geography-course-list | UoL: https://www.liverpool.ac.uk/courses/geography-bsc-hons</t>
+          <t>Host: https://utm.calendar.utoronto.ca/course/ggr387h5 | NEW (Jul 2025 handbook, not previously in this file) - verified in current host catalogue, Oct 2026 | UoL match is a SUGGESTION for department review (programme LOs, not close module match)</t>
         </is>
       </c>
       <c r="K165" s="10" t="inlineStr">
         <is>
-          <t>Original row; Wrong term for partner semester (Fall Semester [Sep-Dec] )</t>
+          <t>Added Oct 2026: July 2025 handbook module verified in current catalogue; UoL match is a suggestion for review; NOT OFFERED 2026/27: Not in the 2026-27 timetable (no Fall 2026 or Winter 2027 section) [https://ttb.utoronto.ca/]</t>
         </is>
       </c>
     </row>
@@ -40313,7 +40313,7 @@
       </c>
       <c r="C166" s="10" t="inlineStr">
         <is>
-          <t>SOES280 HYDROCLIMATE</t>
+          <t>SOES218 GEOMORPHOLOGY: PROCESSES AND FORMS</t>
         </is>
       </c>
       <c r="D166" s="10" t="inlineStr">
@@ -40323,7 +40323,7 @@
       </c>
       <c r="E166" s="10" t="inlineStr">
         <is>
-          <t>GGR214H5 Global Weather and Climate</t>
+          <t>GGR201H5 Introduction to Geomorphology</t>
         </is>
       </c>
       <c r="F166" s="10" t="inlineStr">
@@ -40366,7 +40366,7 @@
       </c>
       <c r="C167" s="10" t="inlineStr">
         <is>
-          <t>SOES218 GEOMORPHOLOGY: PROCESSES AND FORMS</t>
+          <t>SOES280 HYDROCLIMATE</t>
         </is>
       </c>
       <c r="D167" s="10" t="inlineStr">
@@ -40376,12 +40376,12 @@
       </c>
       <c r="E167" s="10" t="inlineStr">
         <is>
-          <t>GGR307H5 Environmental Soil Science (0.5 credit (half course))</t>
+          <t>GGR214H5 Global Weather and Climate</t>
         </is>
       </c>
       <c r="F167" s="10" t="inlineStr">
         <is>
-          <t>Level 3</t>
+          <t>Level 2</t>
         </is>
       </c>
       <c r="G167" s="10" t="inlineStr">
@@ -40391,18 +40391,18 @@
       </c>
       <c r="H167" s="10" t="inlineStr">
         <is>
-          <t>Fall/Winter: check timetable</t>
+          <t>Winter 2027</t>
         </is>
       </c>
       <c r="I167" s="10" t="n"/>
       <c r="J167" s="10" t="inlineStr">
         <is>
-          <t>Host: https://utm.calendar.utoronto.ca/course/ggr307h5 | NEW (Jul 2025 handbook, not previously in this file) - verified in current host catalogue, Oct 2026 | UoL match is a SUGGESTION for department review (programme LOs, not close module match)</t>
+          <t>Host: https://www.utm.utoronto.ca/geography/undergraduate/courses/physical-geography-course-list | UoL: https://www.liverpool.ac.uk/courses/geography-bsc-hons</t>
         </is>
       </c>
       <c r="K167" s="10" t="inlineStr">
         <is>
-          <t>Added Oct 2026: July 2025 handbook module verified in current catalogue; UoL match is a suggestion for review; NOT OFFERED 2026/27: Not in the 2026-27 timetable (no Fall 2026 or Winter 2027 section) [https://ttb.utoronto.ca/]</t>
+          <t>Original row; Wrong term for partner semester (Fall Semester [Sep-Dec] )</t>
         </is>
       </c>
     </row>
@@ -40419,7 +40419,7 @@
       </c>
       <c r="C168" s="10" t="inlineStr">
         <is>
-          <t>SOES280 HYDROCLIMATE</t>
+          <t>SOES218 GEOMORPHOLOGY: PROCESSES AND FORMS</t>
         </is>
       </c>
       <c r="D168" s="10" t="inlineStr">
@@ -40429,7 +40429,7 @@
       </c>
       <c r="E168" s="10" t="inlineStr">
         <is>
-          <t>GGR377H5 Global Climate Change (0.5 credit (half course))</t>
+          <t>GGR307H5 Environmental Soil Science (0.5 credit (half course))</t>
         </is>
       </c>
       <c r="F168" s="10" t="inlineStr">
@@ -40450,29 +40450,29 @@
       <c r="I168" s="10" t="n"/>
       <c r="J168" s="10" t="inlineStr">
         <is>
-          <t>Host: https://utm.calendar.utoronto.ca/course/ggr377h5 | NEW (Jul 2025 handbook, not previously in this file) - verified in current host catalogue, Oct 2026 | UoL match is a SUGGESTION for department review (programme LOs, not close module match)</t>
+          <t>Host: https://utm.calendar.utoronto.ca/course/ggr307h5 | NEW (Jul 2025 handbook, not previously in this file) - verified in current host catalogue, Oct 2026 | UoL match is a SUGGESTION for department review (programme LOs, not close module match)</t>
         </is>
       </c>
       <c r="K168" s="10" t="inlineStr">
         <is>
-          <t>Added Oct 2026: July 2025 handbook module verified in current catalogue; UoL match is a suggestion for review; WRONG TERM 2026/27: Winter 2027 (S) only [https://ttb.utoronto.ca/]</t>
+          <t>Added Oct 2026: July 2025 handbook module verified in current catalogue; UoL match is a suggestion for review; NOT OFFERED 2026/27: Not in the 2026-27 timetable (no Fall 2026 or Winter 2027 section) [https://ttb.utoronto.ca/]</t>
         </is>
       </c>
     </row>
     <row r="169">
       <c r="A169" s="10" t="inlineStr">
         <is>
-          <t>University of Toronto - Scarborough Campus — Canada</t>
+          <t>University of Toronto - Mississauga Campus — Canada</t>
         </is>
       </c>
       <c r="B169" s="10" t="inlineStr">
         <is>
-          <t>Geography BA</t>
+          <t>Geography BSc</t>
         </is>
       </c>
       <c r="C169" s="10" t="inlineStr">
         <is>
-          <t>SOES225 THEMES IN URBAN GEOGRAPHY</t>
+          <t>SOES280 HYDROCLIMATE</t>
         </is>
       </c>
       <c r="D169" s="10" t="inlineStr">
@@ -40482,12 +40482,12 @@
       </c>
       <c r="E169" s="10" t="inlineStr">
         <is>
-          <t>GGRA03H3 Cities and Environments: Urban Life, Livelihoods &amp; Landscapes</t>
+          <t>GGR377H5 Global Climate Change (0.5 credit (half course))</t>
         </is>
       </c>
       <c r="F169" s="10" t="inlineStr">
         <is>
-          <t>Level 1</t>
+          <t>Level 3</t>
         </is>
       </c>
       <c r="G169" s="10" t="inlineStr">
@@ -40497,18 +40497,18 @@
       </c>
       <c r="H169" s="10" t="inlineStr">
         <is>
-          <t>2026/27 catalogue verified; exact term not publicly retrieved</t>
+          <t>Fall/Winter: check timetable</t>
         </is>
       </c>
       <c r="I169" s="10" t="n"/>
       <c r="J169" s="10" t="inlineStr">
         <is>
-          <t>Host: https://www.utsc.utoronto.ca/physsci/environmental-science-course-syllabi | UoL: https://www.liverpool.ac.uk/courses/geography-ba-hons</t>
+          <t>Host: https://utm.calendar.utoronto.ca/course/ggr377h5 | NEW (Jul 2025 handbook, not previously in this file) - verified in current host catalogue, Oct 2026 | UoL match is a SUGGESTION for department review (programme LOs, not close module match)</t>
         </is>
       </c>
       <c r="K169" s="10" t="inlineStr">
         <is>
-          <t>Original row; WRONG TERM 2026/27: Winter 2027 (S) only [https://ttb.utoronto.ca/]</t>
+          <t>Added Oct 2026: July 2025 handbook module verified in current catalogue; UoL match is a suggestion for review; WRONG TERM 2026/27: Winter 2027 (S) only [https://ttb.utoronto.ca/]</t>
         </is>
       </c>
     </row>
@@ -40535,12 +40535,12 @@
       </c>
       <c r="E170" s="10" t="inlineStr">
         <is>
-          <t>GGRB05H3 Urban Geography</t>
+          <t>GGRA03H3 Cities and Environments: Urban Life, Livelihoods &amp; Landscapes</t>
         </is>
       </c>
       <c r="F170" s="10" t="inlineStr">
         <is>
-          <t>Level 2</t>
+          <t>Level 1</t>
         </is>
       </c>
       <c r="G170" s="10" t="inlineStr">
@@ -40561,7 +40561,7 @@
       </c>
       <c r="K170" s="10" t="inlineStr">
         <is>
-          <t>Original row; NOT OFFERED 2026/27: Not in the 2026-27 timetable (no Fall 2026 or Winter 2027 section) [https://ttb.utoronto.ca/]</t>
+          <t>Original row; WRONG TERM 2026/27: Winter 2027 (S) only [https://ttb.utoronto.ca/]</t>
         </is>
       </c>
     </row>
@@ -40578,7 +40578,7 @@
       </c>
       <c r="C171" s="10" t="inlineStr">
         <is>
-          <t>SOES275 SOCIAL AND CULTURAL GEOGRAPHIES</t>
+          <t>SOES225 THEMES IN URBAN GEOGRAPHY</t>
         </is>
       </c>
       <c r="D171" s="10" t="inlineStr">
@@ -40588,7 +40588,7 @@
       </c>
       <c r="E171" s="10" t="inlineStr">
         <is>
-          <t>GGRB13H3 Social Geography: Life and Death, Place and Power</t>
+          <t>GGRB05H3 Urban Geography</t>
         </is>
       </c>
       <c r="F171" s="10" t="inlineStr">
@@ -40641,7 +40641,7 @@
       </c>
       <c r="E172" s="10" t="inlineStr">
         <is>
-          <t>GGRB55H3 Cultural Geography</t>
+          <t>GGRB13H3 Social Geography: Life and Death, Place and Power</t>
         </is>
       </c>
       <c r="F172" s="10" t="inlineStr">
@@ -40694,12 +40694,12 @@
       </c>
       <c r="E173" s="10" t="inlineStr">
         <is>
-          <t>GGRC02H3 Population Geography</t>
+          <t>GGRB55H3 Cultural Geography</t>
         </is>
       </c>
       <c r="F173" s="10" t="inlineStr">
         <is>
-          <t>Level 3</t>
+          <t>Level 2</t>
         </is>
       </c>
       <c r="G173" s="10" t="inlineStr">
@@ -40737,7 +40737,7 @@
       </c>
       <c r="C174" s="10" t="inlineStr">
         <is>
-          <t>SOES225 THEMES IN URBAN GEOGRAPHY</t>
+          <t>SOES275 SOCIAL AND CULTURAL GEOGRAPHIES</t>
         </is>
       </c>
       <c r="D174" s="10" t="inlineStr">
@@ -40747,7 +40747,7 @@
       </c>
       <c r="E174" s="10" t="inlineStr">
         <is>
-          <t>GGRC10H3 Urbanization and Development (0.5 credit (half course))</t>
+          <t>GGRC02H3 Population Geography</t>
         </is>
       </c>
       <c r="F174" s="10" t="inlineStr">
@@ -40762,18 +40762,18 @@
       </c>
       <c r="H174" s="10" t="inlineStr">
         <is>
-          <t>Fall/Winter: check timetable</t>
+          <t>2026/27 catalogue verified; exact term not publicly retrieved</t>
         </is>
       </c>
       <c r="I174" s="10" t="n"/>
       <c r="J174" s="10" t="inlineStr">
         <is>
-          <t>Host: https://utsc.calendar.utoronto.ca/course/ggrc10h3 | NEW (Jul 2025 handbook, not previously in this file) - verified in current host catalogue, Oct 2026 | UoL match is a SUGGESTION for department review (programme LOs, not close module match)</t>
+          <t>Host: https://www.utsc.utoronto.ca/physsci/environmental-science-course-syllabi | UoL: https://www.liverpool.ac.uk/courses/geography-ba-hons</t>
         </is>
       </c>
       <c r="K174" s="10" t="inlineStr">
         <is>
-          <t>Added Oct 2026: July 2025 handbook module verified in current catalogue; UoL match is a suggestion for review; WRONG TERM 2026/27: Winter 2027 (S) only [https://ttb.utoronto.ca/]</t>
+          <t>Original row; NOT OFFERED 2026/27: Not in the 2026-27 timetable (no Fall 2026 or Winter 2027 section) [https://ttb.utoronto.ca/]</t>
         </is>
       </c>
     </row>
@@ -40790,7 +40790,7 @@
       </c>
       <c r="C175" s="10" t="inlineStr">
         <is>
-          <t>SOES270 RETHINKING NATURE: ENVIRONMENTAL KNOWLEDGE, SCIENCE AND SOCIETY</t>
+          <t>SOES225 THEMES IN URBAN GEOGRAPHY</t>
         </is>
       </c>
       <c r="D175" s="10" t="inlineStr">
@@ -40800,7 +40800,7 @@
       </c>
       <c r="E175" s="10" t="inlineStr">
         <is>
-          <t>GGRC26H3 Geographies of Environmental Governance (0.5 credit (half course))</t>
+          <t>GGRC10H3 Urbanization and Development (0.5 credit (half course))</t>
         </is>
       </c>
       <c r="F175" s="10" t="inlineStr">
@@ -40821,12 +40821,12 @@
       <c r="I175" s="10" t="n"/>
       <c r="J175" s="10" t="inlineStr">
         <is>
-          <t>Host: https://utsc.calendar.utoronto.ca/course/ggrc26h3 | NEW (Jul 2025 handbook, not previously in this file) - verified in current host catalogue, Oct 2026 | UoL match is a SUGGESTION for department review (programme LOs, not close module match)</t>
+          <t>Host: https://utsc.calendar.utoronto.ca/course/ggrc10h3 | NEW (Jul 2025 handbook, not previously in this file) - verified in current host catalogue, Oct 2026 | UoL match is a SUGGESTION for department review (programme LOs, not close module match)</t>
         </is>
       </c>
       <c r="K175" s="10" t="inlineStr">
         <is>
-          <t>Added Oct 2026: July 2025 handbook module verified in current catalogue; UoL match is a suggestion for review; NOT OFFERED 2026/27: Not in the 2026-27 timetable (no Fall 2026 or Winter 2027 section) [https://ttb.utoronto.ca/]</t>
+          <t>Added Oct 2026: July 2025 handbook module verified in current catalogue; UoL match is a suggestion for review; WRONG TERM 2026/27: Winter 2027 (S) only [https://ttb.utoronto.ca/]</t>
         </is>
       </c>
     </row>
@@ -40843,7 +40843,7 @@
       </c>
       <c r="C176" s="10" t="inlineStr">
         <is>
-          <t>SOES226 EXPLORING THE SOCIAL WORLD</t>
+          <t>SOES270 RETHINKING NATURE: ENVIRONMENTAL KNOWLEDGE, SCIENCE AND SOCIETY</t>
         </is>
       </c>
       <c r="D176" s="10" t="inlineStr">
@@ -40853,7 +40853,7 @@
       </c>
       <c r="E176" s="10" t="inlineStr">
         <is>
-          <t>GGRC31H3 Qualitative Geographical Methods: Place and Ethnography</t>
+          <t>GGRC26H3 Geographies of Environmental Governance (0.5 credit (half course))</t>
         </is>
       </c>
       <c r="F176" s="10" t="inlineStr">
@@ -40863,23 +40863,23 @@
       </c>
       <c r="G176" s="10" t="inlineStr">
         <is>
-          <t>Core</t>
+          <t>Optional</t>
         </is>
       </c>
       <c r="H176" s="10" t="inlineStr">
         <is>
-          <t>2026/27 catalogue verified; exact term not publicly retrieved</t>
+          <t>Fall/Winter: check timetable</t>
         </is>
       </c>
       <c r="I176" s="10" t="n"/>
       <c r="J176" s="10" t="inlineStr">
         <is>
-          <t>Host: https://www.utsc.utoronto.ca/physsci/environmental-science-course-syllabi | UoL: https://www.liverpool.ac.uk/courses/geography-ba-hons</t>
+          <t>Host: https://utsc.calendar.utoronto.ca/course/ggrc26h3 | NEW (Jul 2025 handbook, not previously in this file) - verified in current host catalogue, Oct 2026 | UoL match is a SUGGESTION for department review (programme LOs, not close module match)</t>
         </is>
       </c>
       <c r="K176" s="10" t="inlineStr">
         <is>
-          <t>Original row; NOT OFFERED 2026/27: Not in the 2026-27 timetable (no Fall 2026 or Winter 2027 section) [https://ttb.utoronto.ca/]</t>
+          <t>Added Oct 2026: July 2025 handbook module verified in current catalogue; UoL match is a suggestion for review; NOT OFFERED 2026/27: Not in the 2026-27 timetable (no Fall 2026 or Winter 2027 section) [https://ttb.utoronto.ca/]</t>
         </is>
       </c>
     </row>
@@ -40891,12 +40891,12 @@
       </c>
       <c r="B177" s="10" t="inlineStr">
         <is>
-          <t>Geography BSc</t>
+          <t>Geography BA</t>
         </is>
       </c>
       <c r="C177" s="10" t="inlineStr">
         <is>
-          <t>SOES214 CHANGING ENVIRONMENTS</t>
+          <t>SOES226 EXPLORING THE SOCIAL WORLD</t>
         </is>
       </c>
       <c r="D177" s="10" t="inlineStr">
@@ -40906,33 +40906,33 @@
       </c>
       <c r="E177" s="10" t="inlineStr">
         <is>
-          <t>EESA06H3 Introduction to Planet Earth</t>
+          <t>GGRC31H3 Qualitative Geographical Methods: Place and Ethnography</t>
         </is>
       </c>
       <c r="F177" s="10" t="inlineStr">
         <is>
-          <t>Level 1</t>
+          <t>Level 3</t>
         </is>
       </c>
       <c r="G177" s="10" t="inlineStr">
         <is>
-          <t>Optional</t>
+          <t>Core</t>
         </is>
       </c>
       <c r="H177" s="10" t="inlineStr">
         <is>
-          <t>Summer 2026 listed; not listed yet for Fall 2026 / Winter 2027</t>
+          <t>2026/27 catalogue verified; exact term not publicly retrieved</t>
         </is>
       </c>
       <c r="I177" s="10" t="n"/>
       <c r="J177" s="10" t="inlineStr">
         <is>
-          <t>Host: https://www.utsc.utoronto.ca/physsci/environmental-science-course-syllabi | UoL: https://www.liverpool.ac.uk/courses/geography-bsc-hons</t>
+          <t>Host: https://www.utsc.utoronto.ca/physsci/environmental-science-course-syllabi | UoL: https://www.liverpool.ac.uk/courses/geography-ba-hons</t>
         </is>
       </c>
       <c r="K177" s="10" t="inlineStr">
         <is>
-          <t>Original row; Workbook semester note says not currently offered</t>
+          <t>Original row; NOT OFFERED 2026/27: Not in the 2026-27 timetable (no Fall 2026 or Winter 2027 section) [https://ttb.utoronto.ca/]</t>
         </is>
       </c>
     </row>
@@ -40959,12 +40959,12 @@
       </c>
       <c r="E178" s="10" t="inlineStr">
         <is>
-          <t>EESB03H3 Principles of Climatology</t>
+          <t>EESA06H3 Introduction to Planet Earth</t>
         </is>
       </c>
       <c r="F178" s="10" t="inlineStr">
         <is>
-          <t>Level 2</t>
+          <t>Level 1</t>
         </is>
       </c>
       <c r="G178" s="10" t="inlineStr">
@@ -41012,7 +41012,7 @@
       </c>
       <c r="E179" s="10" t="inlineStr">
         <is>
-          <t>EESB05H3 Principles of Soil Science</t>
+          <t>EESB03H3 Principles of Climatology</t>
         </is>
       </c>
       <c r="F179" s="10" t="inlineStr">
@@ -41055,7 +41055,7 @@
       </c>
       <c r="C180" s="10" t="inlineStr">
         <is>
-          <t>SOES269 GIS FOR THE NATURAL ENVIRONMENT</t>
+          <t>SOES214 CHANGING ENVIRONMENTS</t>
         </is>
       </c>
       <c r="D180" s="10" t="inlineStr">
@@ -41065,12 +41065,12 @@
       </c>
       <c r="E180" s="10" t="inlineStr">
         <is>
-          <t>EESC03H3 Geographic Information Systems and Remote Sensing</t>
+          <t>EESB05H3 Principles of Soil Science</t>
         </is>
       </c>
       <c r="F180" s="10" t="inlineStr">
         <is>
-          <t>Level 3</t>
+          <t>Level 2</t>
         </is>
       </c>
       <c r="G180" s="10" t="inlineStr">
@@ -41080,7 +41080,7 @@
       </c>
       <c r="H180" s="10" t="inlineStr">
         <is>
-          <t>Not listed for Fall 2026; Winter 2027 schedule not yet populated</t>
+          <t>Summer 2026 listed; not listed yet for Fall 2026 / Winter 2027</t>
         </is>
       </c>
       <c r="I180" s="10" t="n"/>
@@ -41118,12 +41118,12 @@
       </c>
       <c r="E181" s="10" t="inlineStr">
         <is>
-          <t>GGRB32H3 GIS in Action: Processing and Analysis</t>
+          <t>EESC03H3 Geographic Information Systems and Remote Sensing</t>
         </is>
       </c>
       <c r="F181" s="10" t="inlineStr">
         <is>
-          <t>Level 2</t>
+          <t>Level 3</t>
         </is>
       </c>
       <c r="G181" s="10" t="inlineStr">
@@ -41133,7 +41133,7 @@
       </c>
       <c r="H181" s="10" t="inlineStr">
         <is>
-          <t>2026/27 catalogue verified; exact term not publicly retrieved</t>
+          <t>Not listed for Fall 2026; Winter 2027 schedule not yet populated</t>
         </is>
       </c>
       <c r="I181" s="10" t="n"/>
@@ -41144,7 +41144,7 @@
       </c>
       <c r="K181" s="10" t="inlineStr">
         <is>
-          <t>Original row; WRONG TERM 2026/27: Winter 2027 (S) only [https://ttb.utoronto.ca/]</t>
+          <t>Original row; Workbook semester note says not currently offered</t>
         </is>
       </c>
     </row>
@@ -41171,12 +41171,12 @@
       </c>
       <c r="E182" s="10" t="inlineStr">
         <is>
-          <t>GGRC32H3 Essential Spatial Analysis</t>
+          <t>GGRB32H3 GIS in Action: Processing and Analysis</t>
         </is>
       </c>
       <c r="F182" s="10" t="inlineStr">
         <is>
-          <t>Level 3</t>
+          <t>Level 2</t>
         </is>
       </c>
       <c r="G182" s="10" t="inlineStr">
@@ -41204,17 +41204,17 @@
     <row r="183">
       <c r="A183" s="10" t="inlineStr">
         <is>
-          <t>University of Toronto - St. George Campus — Canada</t>
+          <t>University of Toronto - Scarborough Campus — Canada</t>
         </is>
       </c>
       <c r="B183" s="10" t="inlineStr">
         <is>
-          <t>Geography BA</t>
+          <t>Geography BSc</t>
         </is>
       </c>
       <c r="C183" s="10" t="inlineStr">
         <is>
-          <t>SOES225 THEMES IN URBAN GEOGRAPHY</t>
+          <t>SOES269 GIS FOR THE NATURAL ENVIRONMENT</t>
         </is>
       </c>
       <c r="D183" s="10" t="inlineStr">
@@ -41224,7 +41224,7 @@
       </c>
       <c r="E183" s="10" t="inlineStr">
         <is>
-          <t>GGR339H1 Urban Political Geographies</t>
+          <t>GGRC32H3 Essential Spatial Analysis</t>
         </is>
       </c>
       <c r="F183" s="10" t="inlineStr">
@@ -41239,18 +41239,18 @@
       </c>
       <c r="H183" s="10" t="inlineStr">
         <is>
-          <t>2026/27 catalogue verified; exact semester not publicly retrieved</t>
+          <t>2026/27 catalogue verified; exact term not publicly retrieved</t>
         </is>
       </c>
       <c r="I183" s="10" t="n"/>
       <c r="J183" s="10" t="inlineStr">
         <is>
-          <t>Host: https://artsci.calendar.utoronto.ca/section/geography-and-planning | UoL: https://www.liverpool.ac.uk/courses/geography-ba-hons</t>
+          <t>Host: https://www.utsc.utoronto.ca/physsci/environmental-science-course-syllabi | UoL: https://www.liverpool.ac.uk/courses/geography-bsc-hons</t>
         </is>
       </c>
       <c r="K183" s="10" t="inlineStr">
         <is>
-          <t>Original row; NOT OFFERED 2026/27: Not in the 2026-27 timetable (no Fall 2026 or Winter 2027 section) [https://ttb.utoronto.ca/]</t>
+          <t>Original row; WRONG TERM 2026/27: Winter 2027 (S) only [https://ttb.utoronto.ca/]</t>
         </is>
       </c>
     </row>
@@ -41277,12 +41277,12 @@
       </c>
       <c r="E184" s="10" t="inlineStr">
         <is>
-          <t>GGR458H1 Selected Topics in Urban Geography</t>
+          <t>GGR339H1 Urban Political Geographies</t>
         </is>
       </c>
       <c r="F184" s="10" t="inlineStr">
         <is>
-          <t>Upper-level undergraduate</t>
+          <t>Level 3</t>
         </is>
       </c>
       <c r="G184" s="10" t="inlineStr">
@@ -41303,7 +41303,7 @@
       </c>
       <c r="K184" s="10" t="inlineStr">
         <is>
-          <t>Original row; WRONG TERM 2026/27: Winter 2027 (S) only [https://ttb.utoronto.ca/]</t>
+          <t>Original row; NOT OFFERED 2026/27: Not in the 2026-27 timetable (no Fall 2026 or Winter 2027 section) [https://ttb.utoronto.ca/]</t>
         </is>
       </c>
     </row>
@@ -41320,7 +41320,7 @@
       </c>
       <c r="C185" s="10" t="inlineStr">
         <is>
-          <t>SOES222 PLANNING FOR SUSTAINABLE URBANISM</t>
+          <t>SOES225 THEMES IN URBAN GEOGRAPHY</t>
         </is>
       </c>
       <c r="D185" s="10" t="inlineStr">
@@ -41330,7 +41330,7 @@
       </c>
       <c r="E185" s="10" t="inlineStr">
         <is>
-          <t>GGR460H1 Global Cities, Urban Planning, Critical Theory</t>
+          <t>GGR458H1 Selected Topics in Urban Geography</t>
         </is>
       </c>
       <c r="F185" s="10" t="inlineStr">
@@ -41356,7 +41356,7 @@
       </c>
       <c r="K185" s="10" t="inlineStr">
         <is>
-          <t>Original row; NOT OFFERED 2026/27: Not in the 2026-27 timetable (no Fall 2026 or Winter 2027 section) [https://ttb.utoronto.ca/]</t>
+          <t>Original row; WRONG TERM 2026/27: Winter 2027 (S) only [https://ttb.utoronto.ca/]</t>
         </is>
       </c>
     </row>
@@ -41373,7 +41373,7 @@
       </c>
       <c r="C186" s="10" t="inlineStr">
         <is>
-          <t>SOES276 BA GEOGRAPHY EUROPEAN FIELD CLASS</t>
+          <t>SOES222 PLANNING FOR SUSTAINABLE URBANISM</t>
         </is>
       </c>
       <c r="D186" s="10" t="inlineStr">
@@ -41383,7 +41383,7 @@
       </c>
       <c r="E186" s="10" t="inlineStr">
         <is>
-          <t>GGR482H1 Toronto Field Course</t>
+          <t>GGR460H1 Global Cities, Urban Planning, Critical Theory</t>
         </is>
       </c>
       <c r="F186" s="10" t="inlineStr">
@@ -41393,7 +41393,7 @@
       </c>
       <c r="G186" s="10" t="inlineStr">
         <is>
-          <t>Core</t>
+          <t>Optional</t>
         </is>
       </c>
       <c r="H186" s="10" t="inlineStr">
@@ -41426,7 +41426,7 @@
       </c>
       <c r="C187" s="10" t="inlineStr">
         <is>
-          <t>SOES270 RETHINKING NATURE: ENVIRONMENTAL KNOWLEDGE, SCIENCE AND SOCIETY</t>
+          <t>SOES276 BA GEOGRAPHY EUROPEAN FIELD CLASS</t>
         </is>
       </c>
       <c r="D187" s="10" t="inlineStr">
@@ -41436,33 +41436,33 @@
       </c>
       <c r="E187" s="10" t="inlineStr">
         <is>
-          <t>JEG308H1 Canadian Arctic Environments (0.5 credit (half course))</t>
+          <t>GGR482H1 Toronto Field Course</t>
         </is>
       </c>
       <c r="F187" s="10" t="inlineStr">
         <is>
-          <t>Level 3</t>
+          <t>Upper-level undergraduate</t>
         </is>
       </c>
       <c r="G187" s="10" t="inlineStr">
         <is>
-          <t>Optional</t>
+          <t>Core</t>
         </is>
       </c>
       <c r="H187" s="10" t="inlineStr">
         <is>
-          <t>Fall/Winter: check timetable</t>
+          <t>2026/27 catalogue verified; exact semester not publicly retrieved</t>
         </is>
       </c>
       <c r="I187" s="10" t="n"/>
       <c r="J187" s="10" t="inlineStr">
         <is>
-          <t>Host: https://artsci.calendar.utoronto.ca/course/jeg308h1 | NEW (Jul 2025 handbook, not previously in this file) - verified in current host catalogue, Oct 2026 | UoL match is a SUGGESTION for department review (programme LOs, not close module match)</t>
+          <t>Host: https://artsci.calendar.utoronto.ca/section/geography-and-planning | UoL: https://www.liverpool.ac.uk/courses/geography-ba-hons</t>
         </is>
       </c>
       <c r="K187" s="10" t="inlineStr">
         <is>
-          <t>Added Oct 2026: July 2025 handbook module verified in current catalogue; UoL match is a suggestion for review; WRONG TERM 2026/27: Winter 2027 (S) only [https://ttb.utoronto.ca/]</t>
+          <t>Original row; NOT OFFERED 2026/27: Not in the 2026-27 timetable (no Fall 2026 or Winter 2027 section) [https://ttb.utoronto.ca/]</t>
         </is>
       </c>
     </row>
@@ -41474,12 +41474,12 @@
       </c>
       <c r="B188" s="10" t="inlineStr">
         <is>
-          <t>Geography BSc</t>
+          <t>Geography BA</t>
         </is>
       </c>
       <c r="C188" s="10" t="inlineStr">
         <is>
-          <t>SOES269 GIS FOR THE NATURAL ENVIRONMENT</t>
+          <t>SOES270 RETHINKING NATURE: ENVIRONMENTAL KNOWLEDGE, SCIENCE AND SOCIETY</t>
         </is>
       </c>
       <c r="D188" s="10" t="inlineStr">
@@ -41489,12 +41489,12 @@
       </c>
       <c r="E188" s="10" t="inlineStr">
         <is>
-          <t>GGR273H1 Geographic Information and Mapping II</t>
+          <t>JEG308H1 Canadian Arctic Environments (0.5 credit (half course))</t>
         </is>
       </c>
       <c r="F188" s="10" t="inlineStr">
         <is>
-          <t>Level 2</t>
+          <t>Level 3</t>
         </is>
       </c>
       <c r="G188" s="10" t="inlineStr">
@@ -41504,18 +41504,18 @@
       </c>
       <c r="H188" s="10" t="inlineStr">
         <is>
-          <t>2026/27 catalogue verified; exact semester not publicly retrieved</t>
+          <t>Fall/Winter: check timetable</t>
         </is>
       </c>
       <c r="I188" s="10" t="n"/>
       <c r="J188" s="10" t="inlineStr">
         <is>
-          <t>Host: https://artsci.calendar.utoronto.ca/section/geography-and-planning | UoL: https://www.liverpool.ac.uk/courses/geography-bsc-hons</t>
+          <t>Host: https://artsci.calendar.utoronto.ca/course/jeg308h1 | NEW (Jul 2025 handbook, not previously in this file) - verified in current host catalogue, Oct 2026 | UoL match is a SUGGESTION for department review (programme LOs, not close module match)</t>
         </is>
       </c>
       <c r="K188" s="10" t="inlineStr">
         <is>
-          <t>Original row; WRONG TERM 2026/27: Winter 2027 (S) only [https://ttb.utoronto.ca/]</t>
+          <t>Added Oct 2026: July 2025 handbook module verified in current catalogue; UoL match is a suggestion for review; WRONG TERM 2026/27: Winter 2027 (S) only [https://ttb.utoronto.ca/]</t>
         </is>
       </c>
     </row>
@@ -41532,7 +41532,7 @@
       </c>
       <c r="C189" s="10" t="inlineStr">
         <is>
-          <t>SOES214 CHANGING ENVIRONMENTS</t>
+          <t>SOES269 GIS FOR THE NATURAL ENVIRONMENT</t>
         </is>
       </c>
       <c r="D189" s="10" t="inlineStr">
@@ -41542,12 +41542,12 @@
       </c>
       <c r="E189" s="10" t="inlineStr">
         <is>
-          <t>GGR314H1 Global Warming</t>
+          <t>GGR273H1 Geographic Information and Mapping II</t>
         </is>
       </c>
       <c r="F189" s="10" t="inlineStr">
         <is>
-          <t>Level 3</t>
+          <t>Level 2</t>
         </is>
       </c>
       <c r="G189" s="10" t="inlineStr">
@@ -41595,7 +41595,7 @@
       </c>
       <c r="E190" s="10" t="inlineStr">
         <is>
-          <t>GGR348H1 Carbon-Free Energy Systems (0.5 credit (half course))</t>
+          <t>GGR314H1 Global Warming</t>
         </is>
       </c>
       <c r="F190" s="10" t="inlineStr">
@@ -41610,18 +41610,18 @@
       </c>
       <c r="H190" s="10" t="inlineStr">
         <is>
-          <t>Fall/Winter: check timetable</t>
+          <t>2026/27 catalogue verified; exact semester not publicly retrieved</t>
         </is>
       </c>
       <c r="I190" s="10" t="n"/>
       <c r="J190" s="10" t="inlineStr">
         <is>
-          <t>Host: https://artsci.calendar.utoronto.ca/course/ggr348h1 | NEW (Jul 2025 handbook, not previously in this file) - verified in current host catalogue, Oct 2026 | UoL match is a SUGGESTION for department review (programme LOs, not close module match)</t>
+          <t>Host: https://artsci.calendar.utoronto.ca/section/geography-and-planning | UoL: https://www.liverpool.ac.uk/courses/geography-bsc-hons</t>
         </is>
       </c>
       <c r="K190" s="10" t="inlineStr">
         <is>
-          <t>Added Oct 2026: July 2025 handbook module verified in current catalogue; UoL match is a suggestion for review; NOT OFFERED 2026/27: Not in the 2026-27 timetable (no Fall 2026 or Winter 2027 section) [https://ttb.utoronto.ca/]</t>
+          <t>Original row; WRONG TERM 2026/27: Winter 2027 (S) only [https://ttb.utoronto.ca/]</t>
         </is>
       </c>
     </row>
@@ -41638,7 +41638,7 @@
       </c>
       <c r="C191" s="10" t="inlineStr">
         <is>
-          <t>SOES269 GIS FOR THE NATURAL ENVIRONMENT</t>
+          <t>SOES214 CHANGING ENVIRONMENTS</t>
         </is>
       </c>
       <c r="D191" s="10" t="inlineStr">
@@ -41648,7 +41648,7 @@
       </c>
       <c r="E191" s="10" t="inlineStr">
         <is>
-          <t>GGR375H1 Introduction to Programming in GIS</t>
+          <t>GGR348H1 Carbon-Free Energy Systems (0.5 credit (half course))</t>
         </is>
       </c>
       <c r="F191" s="10" t="inlineStr">
@@ -41663,18 +41663,18 @@
       </c>
       <c r="H191" s="10" t="inlineStr">
         <is>
-          <t>2026/27 catalogue verified; exact semester not publicly retrieved</t>
+          <t>Fall/Winter: check timetable</t>
         </is>
       </c>
       <c r="I191" s="10" t="n"/>
       <c r="J191" s="10" t="inlineStr">
         <is>
-          <t>Host: https://artsci.calendar.utoronto.ca/section/geography-and-planning | UoL: https://www.liverpool.ac.uk/courses/geography-bsc-hons</t>
+          <t>Host: https://artsci.calendar.utoronto.ca/course/ggr348h1 | NEW (Jul 2025 handbook, not previously in this file) - verified in current host catalogue, Oct 2026 | UoL match is a SUGGESTION for department review (programme LOs, not close module match)</t>
         </is>
       </c>
       <c r="K191" s="10" t="inlineStr">
         <is>
-          <t>Original row; WRONG TERM 2026/27: Winter 2027 (S) only [https://ttb.utoronto.ca/]</t>
+          <t>Added Oct 2026: July 2025 handbook module verified in current catalogue; UoL match is a suggestion for review; NOT OFFERED 2026/27: Not in the 2026-27 timetable (no Fall 2026 or Winter 2027 section) [https://ttb.utoronto.ca/]</t>
         </is>
       </c>
     </row>
@@ -41691,7 +41691,7 @@
       </c>
       <c r="C192" s="10" t="inlineStr">
         <is>
-          <t>SOES214 CHANGING ENVIRONMENTS</t>
+          <t>SOES269 GIS FOR THE NATURAL ENVIRONMENT</t>
         </is>
       </c>
       <c r="D192" s="10" t="inlineStr">
@@ -41701,7 +41701,7 @@
       </c>
       <c r="E192" s="10" t="inlineStr">
         <is>
-          <t>GGR388H1 Special Topics in Physical &amp; Environmental Geography</t>
+          <t>GGR375H1 Introduction to Programming in GIS</t>
         </is>
       </c>
       <c r="F192" s="10" t="inlineStr">
@@ -41727,24 +41727,24 @@
       </c>
       <c r="K192" s="10" t="inlineStr">
         <is>
-          <t>Original row; NOT OFFERED 2026/27: Not in the 2026-27 timetable (no Fall 2026 or Winter 2027 section) [https://ttb.utoronto.ca/]</t>
+          <t>Original row; WRONG TERM 2026/27: Winter 2027 (S) only [https://ttb.utoronto.ca/]</t>
         </is>
       </c>
     </row>
     <row r="193">
       <c r="A193" s="10" t="inlineStr">
         <is>
-          <t>University of Victoria (UVic) — Canada</t>
+          <t>University of Toronto - St. George Campus — Canada</t>
         </is>
       </c>
       <c r="B193" s="10" t="inlineStr">
         <is>
-          <t>Geography BA</t>
+          <t>Geography BSc</t>
         </is>
       </c>
       <c r="C193" s="10" t="inlineStr">
         <is>
-          <t>SOES224 POLITICAL ECONOMIES OF CRISIS AND CHANGE</t>
+          <t>SOES214 CHANGING ENVIRONMENTS</t>
         </is>
       </c>
       <c r="D193" s="10" t="inlineStr">
@@ -41754,12 +41754,12 @@
       </c>
       <c r="E193" s="10" t="inlineStr">
         <is>
-          <t>GEOG211 Political and Economic Geography</t>
+          <t>GGR388H1 Special Topics in Physical &amp; Environmental Geography</t>
         </is>
       </c>
       <c r="F193" s="10" t="inlineStr">
         <is>
-          <t>Level 2</t>
+          <t>Level 3</t>
         </is>
       </c>
       <c r="G193" s="10" t="inlineStr">
@@ -41769,18 +41769,18 @@
       </c>
       <c r="H193" s="10" t="inlineStr">
         <is>
-          <t>2026/27 module verified; exact Fall/Spring timetable not publicly retrieved</t>
+          <t>2026/27 catalogue verified; exact semester not publicly retrieved</t>
         </is>
       </c>
       <c r="I193" s="10" t="n"/>
       <c r="J193" s="10" t="inlineStr">
         <is>
-          <t>Host: https://www.uvic.ca/socialsciences/geography/programs/ba-bsc-major/index.php | UoL: https://www.liverpool.ac.uk/courses/geography-ba-hons</t>
+          <t>Host: https://artsci.calendar.utoronto.ca/section/geography-and-planning | UoL: https://www.liverpool.ac.uk/courses/geography-bsc-hons</t>
         </is>
       </c>
       <c r="K193" s="10" t="inlineStr">
         <is>
-          <t>Original row; WRONG TERM 2026/27: Spring 2027 only (Second Term) [https://banner.uvic.ca/StudentRegistrationSsb/ssb/classSearch/classSearch]</t>
+          <t>Original row; NOT OFFERED 2026/27: Not in the 2026-27 timetable (no Fall 2026 or Winter 2027 section) [https://ttb.utoronto.ca/]</t>
         </is>
       </c>
     </row>
@@ -41797,7 +41797,7 @@
       </c>
       <c r="C194" s="10" t="inlineStr">
         <is>
-          <t>SOES275 SOCIAL AND CULTURAL GEOGRAPHIES</t>
+          <t>SOES224 POLITICAL ECONOMIES OF CRISIS AND CHANGE</t>
         </is>
       </c>
       <c r="D194" s="10" t="inlineStr">
@@ -41807,7 +41807,7 @@
       </c>
       <c r="E194" s="10" t="inlineStr">
         <is>
-          <t>GEOG218 Social and Cultural Geography</t>
+          <t>GEOG211 Political and Economic Geography</t>
         </is>
       </c>
       <c r="F194" s="10" t="inlineStr">
@@ -41850,7 +41850,7 @@
       </c>
       <c r="C195" s="10" t="inlineStr">
         <is>
-          <t>SOES270 RETHINKING NATURE: ENVIRONMENTAL KNOWLEDGE, SCIENCE AND SOCIETY</t>
+          <t>SOES275 SOCIAL AND CULTURAL GEOGRAPHIES</t>
         </is>
       </c>
       <c r="D195" s="10" t="inlineStr">
@@ -41860,12 +41860,12 @@
       </c>
       <c r="E195" s="10" t="inlineStr">
         <is>
-          <t>GEOG409 Personal Space</t>
+          <t>GEOG218 Social and Cultural Geography</t>
         </is>
       </c>
       <c r="F195" s="10" t="inlineStr">
         <is>
-          <t>Upper-level undergraduate</t>
+          <t>Level 2</t>
         </is>
       </c>
       <c r="G195" s="10" t="inlineStr">
@@ -41898,12 +41898,12 @@
       </c>
       <c r="B196" s="10" t="inlineStr">
         <is>
-          <t>Geography BSc</t>
+          <t>Geography BA</t>
         </is>
       </c>
       <c r="C196" s="10" t="inlineStr">
         <is>
-          <t>SOES280 HYDROCLIMATE</t>
+          <t>SOES270 RETHINKING NATURE: ENVIRONMENTAL KNOWLEDGE, SCIENCE AND SOCIETY</t>
         </is>
       </c>
       <c r="D196" s="10" t="inlineStr">
@@ -41913,12 +41913,12 @@
       </c>
       <c r="E196" s="10" t="inlineStr">
         <is>
-          <t>GEOG130 Climate Change</t>
+          <t>GEOG409 Personal Space</t>
         </is>
       </c>
       <c r="F196" s="10" t="inlineStr">
         <is>
-          <t>Level 1</t>
+          <t>Upper-level undergraduate</t>
         </is>
       </c>
       <c r="G196" s="10" t="inlineStr">
@@ -41934,7 +41934,7 @@
       <c r="I196" s="10" t="n"/>
       <c r="J196" s="10" t="inlineStr">
         <is>
-          <t>Host: https://www.uvic.ca/socialsciences/geography/programs/ba-bsc-major/index.php | UoL: https://www.liverpool.ac.uk/courses/geography-bsc-hons</t>
+          <t>Host: https://www.uvic.ca/socialsciences/geography/programs/ba-bsc-major/index.php | UoL: https://www.liverpool.ac.uk/courses/geography-ba-hons</t>
         </is>
       </c>
       <c r="K196" s="10" t="inlineStr">
@@ -41956,7 +41956,7 @@
       </c>
       <c r="C197" s="10" t="inlineStr">
         <is>
-          <t>SOES213 GEOGRAPHICAL DATA ANALYSIS AND PROCESSING</t>
+          <t>SOES280 HYDROCLIMATE</t>
         </is>
       </c>
       <c r="D197" s="10" t="inlineStr">
@@ -41966,17 +41966,17 @@
       </c>
       <c r="E197" s="10" t="inlineStr">
         <is>
-          <t>GEOG230 Intro to Environmental Data Analysis</t>
+          <t>GEOG130 Climate Change</t>
         </is>
       </c>
       <c r="F197" s="10" t="inlineStr">
         <is>
-          <t>Level 2</t>
+          <t>Level 1</t>
         </is>
       </c>
       <c r="G197" s="10" t="inlineStr">
         <is>
-          <t>Core</t>
+          <t>Optional</t>
         </is>
       </c>
       <c r="H197" s="10" t="inlineStr">
@@ -42009,7 +42009,7 @@
       </c>
       <c r="C198" s="10" t="inlineStr">
         <is>
-          <t>SOES214 CHANGING ENVIRONMENTS</t>
+          <t>SOES213 GEOGRAPHICAL DATA ANALYSIS AND PROCESSING</t>
         </is>
       </c>
       <c r="D198" s="10" t="inlineStr">
@@ -42019,7 +42019,7 @@
       </c>
       <c r="E198" s="10" t="inlineStr">
         <is>
-          <t>GEOG274 Biogeography</t>
+          <t>GEOG230 Intro to Environmental Data Analysis</t>
         </is>
       </c>
       <c r="F198" s="10" t="inlineStr">
@@ -42029,7 +42029,7 @@
       </c>
       <c r="G198" s="10" t="inlineStr">
         <is>
-          <t>Optional</t>
+          <t>Core</t>
         </is>
       </c>
       <c r="H198" s="10" t="inlineStr">
@@ -42062,7 +42062,7 @@
       </c>
       <c r="C199" s="10" t="inlineStr">
         <is>
-          <t>SOES218 GEOMORPHOLOGY: PROCESSES AND FORMS</t>
+          <t>SOES214 CHANGING ENVIRONMENTS</t>
         </is>
       </c>
       <c r="D199" s="10" t="inlineStr">
@@ -42072,7 +42072,7 @@
       </c>
       <c r="E199" s="10" t="inlineStr">
         <is>
-          <t>GEOG276 Geomorphology</t>
+          <t>GEOG274 Biogeography</t>
         </is>
       </c>
       <c r="F199" s="10" t="inlineStr">
@@ -42105,17 +42105,17 @@
     <row r="200">
       <c r="A200" s="10" t="inlineStr">
         <is>
-          <t>University of Waterloo — Canada</t>
+          <t>University of Victoria (UVic) — Canada</t>
         </is>
       </c>
       <c r="B200" s="10" t="inlineStr">
         <is>
-          <t>Geography BA</t>
+          <t>Geography BSc</t>
         </is>
       </c>
       <c r="C200" s="10" t="inlineStr">
         <is>
-          <t>SOES270 RETHINKING NATURE: ENVIRONMENTAL KNOWLEDGE, SCIENCE AND SOCIETY</t>
+          <t>SOES218 GEOMORPHOLOGY: PROCESSES AND FORMS</t>
         </is>
       </c>
       <c r="D200" s="10" t="inlineStr">
@@ -42125,7 +42125,7 @@
       </c>
       <c r="E200" s="10" t="inlineStr">
         <is>
-          <t>GEOG203 Environment and Development in a Global Perspective</t>
+          <t>GEOG276 Geomorphology</t>
         </is>
       </c>
       <c r="F200" s="10" t="inlineStr">
@@ -42140,18 +42140,18 @@
       </c>
       <c r="H200" s="10" t="inlineStr">
         <is>
-          <t>Term not stated in catalogue</t>
+          <t>2026/27 module verified; exact Fall/Spring timetable not publicly retrieved</t>
         </is>
       </c>
       <c r="I200" s="10" t="n"/>
       <c r="J200" s="10" t="inlineStr">
         <is>
-          <t>Host: https://uwaterloocm.kuali.co/ | NEW (Jul 2025 handbook, not previously in this file) - verified in current host catalogue, Oct 2026 | UoL match is a SUGGESTION for department review (programme LOs, not close module match)</t>
+          <t>Host: https://www.uvic.ca/socialsciences/geography/programs/ba-bsc-major/index.php | UoL: https://www.liverpool.ac.uk/courses/geography-bsc-hons</t>
         </is>
       </c>
       <c r="K200" s="10" t="inlineStr">
         <is>
-          <t>Added Oct 2026: July 2025 handbook module verified in current catalogue; UoL match is a suggestion for review; NOT OFFERED 2026/27: No sections Fall 2026 — Course renumbered GEOG 326; no sections listed in Fall 2026 [UW Flow (uwflow.com) section data, term 1269 = Fall 2026]</t>
+          <t>Original row; WRONG TERM 2026/27: Spring 2027 only (Second Term) [https://banner.uvic.ca/StudentRegistrationSsb/ssb/classSearch/classSearch]</t>
         </is>
       </c>
     </row>
@@ -42163,12 +42163,12 @@
       </c>
       <c r="B201" s="10" t="inlineStr">
         <is>
-          <t>Geography BSc</t>
+          <t>Geography BA</t>
         </is>
       </c>
       <c r="C201" s="10" t="inlineStr">
         <is>
-          <t>SOES214 CHANGING ENVIRONMENTS</t>
+          <t>SOES270 RETHINKING NATURE: ENVIRONMENTAL KNOWLEDGE, SCIENCE AND SOCIETY</t>
         </is>
       </c>
       <c r="D201" s="10" t="inlineStr">
@@ -42178,12 +42178,12 @@
       </c>
       <c r="E201" s="10" t="inlineStr">
         <is>
-          <t>GEOG102 Changing Physical Environments</t>
+          <t>GEOG203 Environment and Development in a Global Perspective</t>
         </is>
       </c>
       <c r="F201" s="10" t="inlineStr">
         <is>
-          <t>Level 1</t>
+          <t>Level 2</t>
         </is>
       </c>
       <c r="G201" s="10" t="inlineStr">
@@ -42193,18 +42193,18 @@
       </c>
       <c r="H201" s="10" t="inlineStr">
         <is>
-          <t>Winter 2027 and Spring 2027</t>
+          <t>Term not stated in catalogue</t>
         </is>
       </c>
       <c r="I201" s="10" t="n"/>
       <c r="J201" s="10" t="inlineStr">
         <is>
-          <t>Host: https://classes.uwaterloo.ca/under.html | UoL: https://www.liverpool.ac.uk/courses/geography-bsc-hons</t>
+          <t>Host: https://uwaterloocm.kuali.co/ | NEW (Jul 2025 handbook, not previously in this file) - verified in current host catalogue, Oct 2026 | UoL match is a SUGGESTION for department review (programme LOs, not close module match)</t>
         </is>
       </c>
       <c r="K201" s="10" t="inlineStr">
         <is>
-          <t>Original row; Wrong term for partner semester (Fall Semester [Sep-Dec] )</t>
+          <t>Added Oct 2026: July 2025 handbook module verified in current catalogue; UoL match is a suggestion for review; NOT OFFERED 2026/27: No sections Fall 2026 — Course renumbered GEOG 326; no sections listed in Fall 2026 [UW Flow (uwflow.com) section data, term 1269 = Fall 2026]</t>
         </is>
       </c>
     </row>
@@ -42231,7 +42231,7 @@
       </c>
       <c r="E202" s="10" t="inlineStr">
         <is>
-          <t>GEOG270/AVIA270 RPAS Knowledge Requirements</t>
+          <t>GEOG102 Changing Physical Environments</t>
         </is>
       </c>
       <c r="F202" s="10" t="inlineStr">
@@ -42246,7 +42246,7 @@
       </c>
       <c r="H202" s="10" t="inlineStr">
         <is>
-          <t>Winter 2027</t>
+          <t>Winter 2027 and Spring 2027</t>
         </is>
       </c>
       <c r="I202" s="10" t="n"/>
@@ -42264,17 +42264,17 @@
     <row r="203">
       <c r="A203" s="10" t="inlineStr">
         <is>
-          <t>University of Western Australia — Australia</t>
+          <t>University of Waterloo — Canada</t>
         </is>
       </c>
       <c r="B203" s="10" t="inlineStr">
         <is>
-          <t>Geography BA</t>
+          <t>Geography BSc</t>
         </is>
       </c>
       <c r="C203" s="10" t="inlineStr">
         <is>
-          <t>SOES270 RETHINKING NATURE: ENVIRONMENTAL KNOWLEDGE, SCIENCE AND SOCIETY</t>
+          <t>SOES214 CHANGING ENVIRONMENTS</t>
         </is>
       </c>
       <c r="D203" s="10" t="inlineStr">
@@ -42284,12 +42284,12 @@
       </c>
       <c r="E203" s="10" t="inlineStr">
         <is>
-          <t>GEOG2202 Reading Landscapes: People and Processes</t>
+          <t>GEOG270/AVIA270 RPAS Knowledge Requirements</t>
         </is>
       </c>
       <c r="F203" s="10" t="inlineStr">
         <is>
-          <t>Level 2</t>
+          <t>Level 1</t>
         </is>
       </c>
       <c r="G203" s="10" t="inlineStr">
@@ -42299,18 +42299,18 @@
       </c>
       <c r="H203" s="10" t="inlineStr">
         <is>
-          <t>Semester 2 (2026)</t>
+          <t>Winter 2027</t>
         </is>
       </c>
       <c r="I203" s="10" t="n"/>
       <c r="J203" s="10" t="inlineStr">
         <is>
-          <t>Host: https://handbooks.uwa.edu.au/ | UoL: https://www.liverpool.ac.uk/courses/geography-ba-hons</t>
+          <t>Host: https://classes.uwaterloo.ca/under.html | UoL: https://www.liverpool.ac.uk/courses/geography-bsc-hons</t>
         </is>
       </c>
       <c r="K203" s="10" t="inlineStr">
         <is>
-          <t>Original row; Wrong term for partner semester (Semester 1)</t>
+          <t>Original row; Wrong term for partner semester (Fall Semester [Sep-Dec] )</t>
         </is>
       </c>
     </row>
@@ -42327,7 +42327,7 @@
       </c>
       <c r="C204" s="10" t="inlineStr">
         <is>
-          <t>SOES220 CITIES AND REGIONS</t>
+          <t>SOES270 RETHINKING NATURE: ENVIRONMENTAL KNOWLEDGE, SCIENCE AND SOCIETY</t>
         </is>
       </c>
       <c r="D204" s="10" t="inlineStr">
@@ -42337,7 +42337,7 @@
       </c>
       <c r="E204" s="10" t="inlineStr">
         <is>
-          <t>GEOG2203 Regions in Transition</t>
+          <t>GEOG2202 Reading Landscapes: People and Processes</t>
         </is>
       </c>
       <c r="F204" s="10" t="inlineStr">
@@ -42380,7 +42380,7 @@
       </c>
       <c r="C205" s="10" t="inlineStr">
         <is>
-          <t>SOES270 RETHINKING NATURE: ENVIRONMENTAL KNOWLEDGE, SCIENCE AND SOCIETY</t>
+          <t>SOES220 CITIES AND REGIONS</t>
         </is>
       </c>
       <c r="D205" s="10" t="inlineStr">
@@ -42390,12 +42390,12 @@
       </c>
       <c r="E205" s="10" t="inlineStr">
         <is>
-          <t>GEOG3312 Migrants, Refugees and Borders</t>
+          <t>GEOG2203 Regions in Transition</t>
         </is>
       </c>
       <c r="F205" s="10" t="inlineStr">
         <is>
-          <t>Level 3</t>
+          <t>Level 2</t>
         </is>
       </c>
       <c r="G205" s="10" t="inlineStr">
@@ -42428,12 +42428,12 @@
       </c>
       <c r="B206" s="10" t="inlineStr">
         <is>
-          <t>Geography BSc</t>
+          <t>Geography BA</t>
         </is>
       </c>
       <c r="C206" s="10" t="inlineStr">
         <is>
-          <t>SOES280 HYDROCLIMATE</t>
+          <t>SOES270 RETHINKING NATURE: ENVIRONMENTAL KNOWLEDGE, SCIENCE AND SOCIETY</t>
         </is>
       </c>
       <c r="D206" s="10" t="inlineStr">
@@ -42443,12 +42443,12 @@
       </c>
       <c r="E206" s="10" t="inlineStr">
         <is>
-          <t>ENVT2251 Hydrology and Water Resource Management</t>
+          <t>GEOG3312 Migrants, Refugees and Borders</t>
         </is>
       </c>
       <c r="F206" s="10" t="inlineStr">
         <is>
-          <t>Level 2</t>
+          <t>Level 3</t>
         </is>
       </c>
       <c r="G206" s="10" t="inlineStr">
@@ -42464,7 +42464,7 @@
       <c r="I206" s="10" t="n"/>
       <c r="J206" s="10" t="inlineStr">
         <is>
-          <t>Host: https://handbooks.uwa.edu.au/ | UoL: https://www.liverpool.ac.uk/courses/geography-bsc-hons</t>
+          <t>Host: https://handbooks.uwa.edu.au/ | UoL: https://www.liverpool.ac.uk/courses/geography-ba-hons</t>
         </is>
       </c>
       <c r="K206" s="10" t="inlineStr">
@@ -42486,7 +42486,7 @@
       </c>
       <c r="C207" s="10" t="inlineStr">
         <is>
-          <t>SOES269 GIS FOR THE NATURAL ENVIRONMENT</t>
+          <t>SOES280 HYDROCLIMATE</t>
         </is>
       </c>
       <c r="D207" s="10" t="inlineStr">
@@ -42496,12 +42496,12 @@
       </c>
       <c r="E207" s="10" t="inlineStr">
         <is>
-          <t>GEOG3301 Advanced GIS and Remote Sensing</t>
+          <t>ENVT2251 Hydrology and Water Resource Management</t>
         </is>
       </c>
       <c r="F207" s="10" t="inlineStr">
         <is>
-          <t>Level 3</t>
+          <t>Level 2</t>
         </is>
       </c>
       <c r="G207" s="10" t="inlineStr">
@@ -42539,7 +42539,7 @@
       </c>
       <c r="C208" s="10" t="inlineStr">
         <is>
-          <t>SOES225 THEMES IN URBAN GEOGRAPHY</t>
+          <t>SOES269 GIS FOR THE NATURAL ENVIRONMENT</t>
         </is>
       </c>
       <c r="D208" s="10" t="inlineStr">
@@ -42549,7 +42549,7 @@
       </c>
       <c r="E208" s="10" t="inlineStr">
         <is>
-          <t>GEOG3303 Environmental Policy and Planning</t>
+          <t>GEOG3301 Advanced GIS and Remote Sensing</t>
         </is>
       </c>
       <c r="F208" s="10" t="inlineStr">
@@ -42582,17 +42582,17 @@
     <row r="209">
       <c r="A209" s="10" t="inlineStr">
         <is>
-          <t>University of Wollongong — Australia</t>
+          <t>University of Western Australia — Australia</t>
         </is>
       </c>
       <c r="B209" s="10" t="inlineStr">
         <is>
-          <t>Geography BA</t>
+          <t>Geography BSc</t>
         </is>
       </c>
       <c r="C209" s="10" t="inlineStr">
         <is>
-          <t>SOES275 SOCIAL AND CULTURAL GEOGRAPHIES</t>
+          <t>SOES225 THEMES IN URBAN GEOGRAPHY</t>
         </is>
       </c>
       <c r="D209" s="10" t="inlineStr">
@@ -42602,12 +42602,12 @@
       </c>
       <c r="E209" s="10" t="inlineStr">
         <is>
-          <t>GEOG222 Society and Environment: Resources, Challenges, Futures (6 CP)</t>
+          <t>GEOG3303 Environmental Policy and Planning</t>
         </is>
       </c>
       <c r="F209" s="10" t="inlineStr">
         <is>
-          <t>Level 2</t>
+          <t>Level 3</t>
         </is>
       </c>
       <c r="G209" s="10" t="inlineStr">
@@ -42617,18 +42617,18 @@
       </c>
       <c r="H209" s="10" t="inlineStr">
         <is>
-          <t>Spring</t>
+          <t>Semester 2 (2026)</t>
         </is>
       </c>
       <c r="I209" s="10" t="n"/>
       <c r="J209" s="10" t="inlineStr">
         <is>
-          <t>Host: https://courses.uow.edu.au/courses/2026/1708 | UoL: https://www.liverpool.ac.uk/courses/geography-ba-hons</t>
+          <t>Host: https://handbooks.uwa.edu.au/ | UoL: https://www.liverpool.ac.uk/courses/geography-bsc-hons</t>
         </is>
       </c>
       <c r="K209" s="10" t="inlineStr">
         <is>
-          <t>Original row; Wrong term for partner semester (Autumn Semester (Feb-Jul))</t>
+          <t>Original row; Wrong term for partner semester (Semester 1)</t>
         </is>
       </c>
     </row>
@@ -42645,7 +42645,7 @@
       </c>
       <c r="C210" s="10" t="inlineStr">
         <is>
-          <t>SOES270 RETHINKING NATURE: ENVIRONMENTAL KNOWLEDGE, SCIENCE AND SOCIETY</t>
+          <t>SOES275 SOCIAL AND CULTURAL GEOGRAPHIES</t>
         </is>
       </c>
       <c r="D210" s="10" t="inlineStr">
@@ -42655,7 +42655,7 @@
       </c>
       <c r="E210" s="10" t="inlineStr">
         <is>
-          <t>GEOG224 Future of Food (6 CP)</t>
+          <t>GEOG222 Society and Environment: Resources, Challenges, Futures (6 CP)</t>
         </is>
       </c>
       <c r="F210" s="10" t="inlineStr">
@@ -42698,7 +42698,7 @@
       </c>
       <c r="C211" s="10" t="inlineStr">
         <is>
-          <t>SOES277 GIS FOR SOCIAL SCIENCES</t>
+          <t>SOES270 RETHINKING NATURE: ENVIRONMENTAL KNOWLEDGE, SCIENCE AND SOCIETY</t>
         </is>
       </c>
       <c r="D211" s="10" t="inlineStr">
@@ -42708,7 +42708,7 @@
       </c>
       <c r="E211" s="10" t="inlineStr">
         <is>
-          <t>GEOG231 Maps, Apps and Spatial Media (6 CP)</t>
+          <t>GEOG224 Future of Food (6 CP)</t>
         </is>
       </c>
       <c r="F211" s="10" t="inlineStr">
@@ -42746,12 +42746,12 @@
       </c>
       <c r="B212" s="10" t="inlineStr">
         <is>
-          <t>Geography BSc</t>
+          <t>Geography BA</t>
         </is>
       </c>
       <c r="C212" s="10" t="inlineStr">
         <is>
-          <t>SOES214 CHANGING ENVIRONMENTS</t>
+          <t>SOES277 GIS FOR SOCIAL SCIENCES</t>
         </is>
       </c>
       <c r="D212" s="10" t="inlineStr">
@@ -42761,12 +42761,12 @@
       </c>
       <c r="E212" s="10" t="inlineStr">
         <is>
-          <t>EESC202 Shaping Earth’s Surface (6 CP)</t>
+          <t>GEOG231 Maps, Apps and Spatial Media (6 CP)</t>
         </is>
       </c>
       <c r="F212" s="10" t="inlineStr">
         <is>
-          <t>Level 3</t>
+          <t>Level 2</t>
         </is>
       </c>
       <c r="G212" s="10" t="inlineStr">
@@ -42782,7 +42782,7 @@
       <c r="I212" s="10" t="n"/>
       <c r="J212" s="10" t="inlineStr">
         <is>
-          <t>Host: https://courses.uow.edu.au/courses/2026/1708 | UoL: https://www.liverpool.ac.uk/courses/geography-bsc-hons</t>
+          <t>Host: https://courses.uow.edu.au/courses/2026/1708 | UoL: https://www.liverpool.ac.uk/courses/geography-ba-hons</t>
         </is>
       </c>
       <c r="K212" s="10" t="inlineStr">
@@ -42804,7 +42804,7 @@
       </c>
       <c r="C213" s="10" t="inlineStr">
         <is>
-          <t>SOES269 GIS FOR THE NATURAL ENVIRONMENT</t>
+          <t>SOES214 CHANGING ENVIRONMENTS</t>
         </is>
       </c>
       <c r="D213" s="10" t="inlineStr">
@@ -42814,7 +42814,7 @@
       </c>
       <c r="E213" s="10" t="inlineStr">
         <is>
-          <t>EESC207 Advanced Geospatial Analysis (6 CP)</t>
+          <t>EESC202 Shaping Earth’s Surface (6 CP)</t>
         </is>
       </c>
       <c r="F213" s="10" t="inlineStr">
@@ -42829,18 +42829,18 @@
       </c>
       <c r="H213" s="10" t="inlineStr">
         <is>
-          <t>Not available for new enrolments from 2026</t>
+          <t>Spring</t>
         </is>
       </c>
       <c r="I213" s="10" t="n"/>
       <c r="J213" s="10" t="inlineStr">
         <is>
-          <t>Host: https://courses.uow.edu.au/subjects/2026/EESC207 | UoL: https://www.liverpool.ac.uk/courses/geography-bsc-hons</t>
+          <t>Host: https://courses.uow.edu.au/courses/2026/1708 | UoL: https://www.liverpool.ac.uk/courses/geography-bsc-hons</t>
         </is>
       </c>
       <c r="K213" s="10" t="inlineStr">
         <is>
-          <t>Original row; Workbook semester note says not currently offered</t>
+          <t>Original row; Wrong term for partner semester (Autumn Semester (Feb-Jul))</t>
         </is>
       </c>
     </row>
@@ -42857,7 +42857,7 @@
       </c>
       <c r="C214" s="10" t="inlineStr">
         <is>
-          <t>SOES214 CHANGING ENVIRONMENTS</t>
+          <t>SOES269 GIS FOR THE NATURAL ENVIRONMENT</t>
         </is>
       </c>
       <c r="D214" s="10" t="inlineStr">
@@ -42867,12 +42867,12 @@
       </c>
       <c r="E214" s="10" t="inlineStr">
         <is>
-          <t>GEOG231 Maps, Apps and Spatial Media (6 CP)</t>
+          <t>EESC207 Advanced Geospatial Analysis (6 CP)</t>
         </is>
       </c>
       <c r="F214" s="10" t="inlineStr">
         <is>
-          <t>Level 2</t>
+          <t>Level 3</t>
         </is>
       </c>
       <c r="G214" s="10" t="inlineStr">
@@ -42882,18 +42882,18 @@
       </c>
       <c r="H214" s="10" t="inlineStr">
         <is>
-          <t>Spring</t>
+          <t>Not available for new enrolments from 2026</t>
         </is>
       </c>
       <c r="I214" s="10" t="n"/>
       <c r="J214" s="10" t="inlineStr">
         <is>
-          <t>Host: https://courses.uow.edu.au/courses/2026/1708 | UoL: https://www.liverpool.ac.uk/courses/geography-bsc-hons</t>
+          <t>Host: https://courses.uow.edu.au/subjects/2026/EESC207 | UoL: https://www.liverpool.ac.uk/courses/geography-bsc-hons</t>
         </is>
       </c>
       <c r="K214" s="10" t="inlineStr">
         <is>
-          <t>Original row; Wrong term for partner semester (Autumn Semester (Feb-Jul))</t>
+          <t>Original row; Workbook semester note says not currently offered</t>
         </is>
       </c>
     </row>
@@ -42910,7 +42910,7 @@
       </c>
       <c r="C215" s="10" t="inlineStr">
         <is>
-          <t>SOES269 GIS FOR THE NATURAL ENVIRONMENT</t>
+          <t>SOES214 CHANGING ENVIRONMENTS</t>
         </is>
       </c>
       <c r="D215" s="10" t="inlineStr">
@@ -42920,12 +42920,12 @@
       </c>
       <c r="E215" s="10" t="inlineStr">
         <is>
-          <t>SCII310 Remote Sensing (6 CP)</t>
+          <t>GEOG231 Maps, Apps and Spatial Media (6 CP)</t>
         </is>
       </c>
       <c r="F215" s="10" t="inlineStr">
         <is>
-          <t>Level 3</t>
+          <t>Level 2</t>
         </is>
       </c>
       <c r="G215" s="10" t="inlineStr">
@@ -42935,7 +42935,7 @@
       </c>
       <c r="H215" s="10" t="inlineStr">
         <is>
-          <t>Autumn</t>
+          <t>Spring</t>
         </is>
       </c>
       <c r="I215" s="10" t="n"/>
@@ -42946,24 +42946,24 @@
       </c>
       <c r="K215" s="10" t="inlineStr">
         <is>
-          <t>Original row; Verified Oct 2026: No teaching periods in 2026 or 2027 - not offered (verified Oct 2026)</t>
+          <t>Original row; Wrong term for partner semester (Autumn Semester (Feb-Jul))</t>
         </is>
       </c>
     </row>
     <row r="216">
       <c r="A216" s="10" t="inlineStr">
         <is>
-          <t>Victoria University of Wellington — New Zealand</t>
+          <t>University of Wollongong — Australia</t>
         </is>
       </c>
       <c r="B216" s="10" t="inlineStr">
         <is>
-          <t>Geography BA</t>
+          <t>Geography BSc</t>
         </is>
       </c>
       <c r="C216" s="10" t="inlineStr">
         <is>
-          <t>SOES270 RETHINKING NATURE: ENVIRONMENTAL KNOWLEDGE, SCIENCE AND SOCIETY</t>
+          <t>SOES269 GIS FOR THE NATURAL ENVIRONMENT</t>
         </is>
       </c>
       <c r="D216" s="10" t="inlineStr">
@@ -42973,12 +42973,12 @@
       </c>
       <c r="E216" s="10" t="inlineStr">
         <is>
-          <t>GEOG217 Human Geography: Approaching Our World (20 points)</t>
+          <t>SCII310 Remote Sensing (6 CP)</t>
         </is>
       </c>
       <c r="F216" s="10" t="inlineStr">
         <is>
-          <t>Level 2</t>
+          <t>Level 3</t>
         </is>
       </c>
       <c r="G216" s="10" t="inlineStr">
@@ -42988,18 +42988,18 @@
       </c>
       <c r="H216" s="10" t="inlineStr">
         <is>
-          <t>2026 course verified; exact trimester not publicly specified</t>
+          <t>Autumn</t>
         </is>
       </c>
       <c r="I216" s="10" t="n"/>
       <c r="J216" s="10" t="inlineStr">
         <is>
-          <t>Host: https://www.wgtn.ac.nz/study/programmes-courses/courses/by-subject?sub=59 | UoL: https://www.liverpool.ac.uk/courses/geography-ba-hons</t>
+          <t>Host: https://courses.uow.edu.au/courses/2026/1708 | UoL: https://www.liverpool.ac.uk/courses/geography-bsc-hons</t>
         </is>
       </c>
       <c r="K216" s="10" t="inlineStr">
         <is>
-          <t>Original row; Verified Oct 2026: Trimester 2 only (2026, 2027) - verified Oct 2026</t>
+          <t>Original row; Verified Oct 2026: No teaching periods in 2026 or 2027 - not offered (verified Oct 2026)</t>
         </is>
       </c>
     </row>
@@ -43016,7 +43016,7 @@
       </c>
       <c r="C217" s="10" t="inlineStr">
         <is>
-          <t>SOES276 BA GEOGRAPHY EUROPEAN FIELD CLASS</t>
+          <t>SOES270 RETHINKING NATURE: ENVIRONMENTAL KNOWLEDGE, SCIENCE AND SOCIETY</t>
         </is>
       </c>
       <c r="D217" s="10" t="inlineStr">
@@ -43026,17 +43026,17 @@
       </c>
       <c r="E217" s="10" t="inlineStr">
         <is>
-          <t>GEOG327 Research Project: Fieldwork and Analysis (20 points)</t>
+          <t>GEOG217 Human Geography: Approaching Our World (20 points)</t>
         </is>
       </c>
       <c r="F217" s="10" t="inlineStr">
         <is>
-          <t>Level 3</t>
+          <t>Level 2</t>
         </is>
       </c>
       <c r="G217" s="10" t="inlineStr">
         <is>
-          <t>Core</t>
+          <t>Optional</t>
         </is>
       </c>
       <c r="H217" s="10" t="inlineStr">
@@ -43064,12 +43064,12 @@
       </c>
       <c r="B218" s="10" t="inlineStr">
         <is>
-          <t>Geography BSc</t>
+          <t>Geography BA</t>
         </is>
       </c>
       <c r="C218" s="10" t="inlineStr">
         <is>
-          <t>SOES214 CHANGING ENVIRONMENTS</t>
+          <t>SOES276 BA GEOGRAPHY EUROPEAN FIELD CLASS</t>
         </is>
       </c>
       <c r="D218" s="10" t="inlineStr">
@@ -43079,28 +43079,28 @@
       </c>
       <c r="E218" s="10" t="inlineStr">
         <is>
-          <t>GEOG214 Environmental Futures for Aotearoa New Zealand (20 points)</t>
+          <t>GEOG327 Research Project: Fieldwork and Analysis (20 points)</t>
         </is>
       </c>
       <c r="F218" s="10" t="inlineStr">
         <is>
-          <t>Level 2</t>
+          <t>Level 3</t>
         </is>
       </c>
       <c r="G218" s="10" t="inlineStr">
         <is>
-          <t>Optional</t>
+          <t>Core</t>
         </is>
       </c>
       <c r="H218" s="10" t="inlineStr">
         <is>
-          <t>Trimester 2 (2026)</t>
+          <t>2026 course verified; exact trimester not publicly specified</t>
         </is>
       </c>
       <c r="I218" s="10" t="n"/>
       <c r="J218" s="10" t="inlineStr">
         <is>
-          <t>Host: https://www.wgtn.ac.nz/study/programmes-courses/courses/by-subject?sub=59 | UoL: https://www.liverpool.ac.uk/courses/geography-bsc-hons</t>
+          <t>Host: https://www.wgtn.ac.nz/study/programmes-courses/courses/by-subject?sub=59 | UoL: https://www.liverpool.ac.uk/courses/geography-ba-hons</t>
         </is>
       </c>
       <c r="K218" s="10" t="inlineStr">
@@ -43122,7 +43122,7 @@
       </c>
       <c r="C219" s="10" t="inlineStr">
         <is>
-          <t>SOES269 GIS FOR THE NATURAL ENVIRONMENT</t>
+          <t>SOES214 CHANGING ENVIRONMENTS</t>
         </is>
       </c>
       <c r="D219" s="10" t="inlineStr">
@@ -43132,7 +43132,7 @@
       </c>
       <c r="E219" s="10" t="inlineStr">
         <is>
-          <t>GEOG215 Introduction to GIS and Science (20 points)</t>
+          <t>GEOG214 Environmental Futures for Aotearoa New Zealand (20 points)</t>
         </is>
       </c>
       <c r="F219" s="10" t="inlineStr">
@@ -43147,7 +43147,7 @@
       </c>
       <c r="H219" s="10" t="inlineStr">
         <is>
-          <t>2026 course verified; exact trimester not publicly specified</t>
+          <t>Trimester 2 (2026)</t>
         </is>
       </c>
       <c r="I219" s="10" t="n"/>
@@ -43185,12 +43185,12 @@
       </c>
       <c r="E220" s="10" t="inlineStr">
         <is>
-          <t>GEOG415 Introduction to GIS and Applications (20 points)</t>
+          <t>GEOG215 Introduction to GIS and Science (20 points)</t>
         </is>
       </c>
       <c r="F220" s="10" t="inlineStr">
         <is>
-          <t>Upper-level undergraduate</t>
+          <t>Level 2</t>
         </is>
       </c>
       <c r="G220" s="10" t="inlineStr">
@@ -43211,7 +43211,7 @@
       </c>
       <c r="K220" s="10" t="inlineStr">
         <is>
-          <t>Original row; WRONG TERM 2026/27: Trimester 2 2027 [https://www.wgtn.ac.nz/courses/geog/415/2027]</t>
+          <t>Original row; Verified Oct 2026: Trimester 2 only (2026, 2027) - verified Oct 2026</t>
         </is>
       </c>
     </row>
@@ -43228,7 +43228,7 @@
       </c>
       <c r="C221" s="10" t="inlineStr">
         <is>
-          <t>SOES280 HYDROCLIMATE</t>
+          <t>SOES269 GIS FOR THE NATURAL ENVIRONMENT</t>
         </is>
       </c>
       <c r="D221" s="10" t="inlineStr">
@@ -43238,12 +43238,12 @@
       </c>
       <c r="E221" s="10" t="inlineStr">
         <is>
-          <t>GEOS301 Hydrological Science &amp; Freshwater Management</t>
+          <t>GEOG415 Introduction to GIS and Applications (20 points)</t>
         </is>
       </c>
       <c r="F221" s="10" t="inlineStr">
         <is>
-          <t>Level 3</t>
+          <t>Upper-level undergraduate</t>
         </is>
       </c>
       <c r="G221" s="10" t="inlineStr">
@@ -43253,7 +43253,7 @@
       </c>
       <c r="H221" s="10" t="inlineStr">
         <is>
-          <t>Not offered in 2026</t>
+          <t>2026 course verified; exact trimester not publicly specified</t>
         </is>
       </c>
       <c r="I221" s="10" t="n"/>
@@ -43264,14 +43264,14 @@
       </c>
       <c r="K221" s="10" t="inlineStr">
         <is>
-          <t>Original row; Workbook semester note says not currently offered</t>
+          <t>Original row; WRONG TERM 2026/27: Trimester 2 2027 [https://www.wgtn.ac.nz/courses/geog/415/2027]</t>
         </is>
       </c>
     </row>
     <row r="222">
       <c r="A222" s="10" t="inlineStr">
         <is>
-          <t>Washington State University — USA</t>
+          <t>Victoria University of Wellington — New Zealand</t>
         </is>
       </c>
       <c r="B222" s="10" t="inlineStr">
@@ -43281,7 +43281,7 @@
       </c>
       <c r="C222" s="10" t="inlineStr">
         <is>
-          <t>SOES214 CHANGING ENVIRONMENTS</t>
+          <t>SOES280 HYDROCLIMATE</t>
         </is>
       </c>
       <c r="D222" s="10" t="inlineStr">
@@ -43291,7 +43291,7 @@
       </c>
       <c r="E222" s="10" t="inlineStr">
         <is>
-          <t>SOC331 Population, Resources, and the Future</t>
+          <t>GEOS301 Hydrological Science &amp; Freshwater Management</t>
         </is>
       </c>
       <c r="F222" s="10" t="inlineStr">
@@ -43306,18 +43306,18 @@
       </c>
       <c r="H222" s="10" t="inlineStr">
         <is>
-          <t>Term not stated in catalogue</t>
+          <t>Not offered in 2026</t>
         </is>
       </c>
       <c r="I222" s="10" t="n"/>
       <c r="J222" s="10" t="inlineStr">
         <is>
-          <t>Host: https://catalog.wsu.edu/Pullman/Academics/Courses/SOC | NEW (Jul 2025 handbook, not previously in this file) - verified in current host catalogue, Oct 2026 via web search | UoL match is a SUGGESTION for department review (programme LOs, not close module match)</t>
+          <t>Host: https://www.wgtn.ac.nz/study/programmes-courses/courses/by-subject?sub=59 | UoL: https://www.liverpool.ac.uk/courses/geography-bsc-hons</t>
         </is>
       </c>
       <c r="K222" s="10" t="inlineStr">
         <is>
-          <t>Added Oct 2026: July 2025 handbook module verified in current catalogue; UoL match is a suggestion for review; NOT OFFERED 2026/27: Not in Fall 2026 Pullman schedule [https://schedules.wsu.edu/ (Schedule of Classes, Fall 2026, Pullman)]</t>
+          <t>Original row; Workbook semester note says not currently offered</t>
         </is>
       </c>
     </row>
@@ -43344,12 +43344,12 @@
       </c>
       <c r="E223" s="10" t="inlineStr">
         <is>
-          <t>SOE 102 Physical Geology</t>
+          <t>SOC331 Population, Resources, and the Future</t>
         </is>
       </c>
       <c r="F223" s="10" t="inlineStr">
         <is>
-          <t>Level 1</t>
+          <t>Level 3</t>
         </is>
       </c>
       <c r="G223" s="10" t="inlineStr">
@@ -43359,18 +43359,18 @@
       </c>
       <c r="H223" s="10" t="inlineStr">
         <is>
-          <t>2026/27 course verified; exact section term not publicly retrieved</t>
+          <t>Term not stated in catalogue</t>
         </is>
       </c>
       <c r="I223" s="10" t="n"/>
       <c r="J223" s="10" t="inlineStr">
         <is>
-          <t>Host: https://environment.wsu.edu/undergraduate-studies/bs-in-earth-and-environmental-sciences/earth-science/ | UoL: https://www.liverpool.ac.uk/courses/geography-bsc-hons</t>
+          <t>Host: https://catalog.wsu.edu/Pullman/Academics/Courses/SOC | NEW (Jul 2025 handbook, not previously in this file) - verified in current host catalogue, Oct 2026 via web search | UoL match is a SUGGESTION for department review (programme LOs, not close module match)</t>
         </is>
       </c>
       <c r="K223" s="10" t="inlineStr">
         <is>
-          <t>Original row; NOT OFFERED 2026/27: Not in Fall 2026 Pullman schedule [https://schedules.wsu.edu/ (Schedule of Classes, Fall 2026, Pullman)]</t>
+          <t>Added Oct 2026: July 2025 handbook module verified in current catalogue; UoL match is a suggestion for review; NOT OFFERED 2026/27: Not in Fall 2026 Pullman schedule [https://schedules.wsu.edu/ (Schedule of Classes, Fall 2026, Pullman)]</t>
         </is>
       </c>
     </row>
@@ -43397,12 +43397,12 @@
       </c>
       <c r="E224" s="10" t="inlineStr">
         <is>
-          <t>SOE 250 Introduction to Earth System Science</t>
+          <t>SOE 102 Physical Geology</t>
         </is>
       </c>
       <c r="F224" s="10" t="inlineStr">
         <is>
-          <t>Level 2</t>
+          <t>Level 1</t>
         </is>
       </c>
       <c r="G224" s="10" t="inlineStr">
@@ -43440,7 +43440,7 @@
       </c>
       <c r="C225" s="10" t="inlineStr">
         <is>
-          <t>SOES269 GIS FOR THE NATURAL ENVIRONMENT</t>
+          <t>SOES214 CHANGING ENVIRONMENTS</t>
         </is>
       </c>
       <c r="D225" s="10" t="inlineStr">
@@ -43450,12 +43450,12 @@
       </c>
       <c r="E225" s="10" t="inlineStr">
         <is>
-          <t>SOE 486 Applied Remote Sensing: From Drones to Satellites</t>
+          <t>SOE 250 Introduction to Earth System Science</t>
         </is>
       </c>
       <c r="F225" s="10" t="inlineStr">
         <is>
-          <t>Upper-level undergraduate</t>
+          <t>Level 2</t>
         </is>
       </c>
       <c r="G225" s="10" t="inlineStr">
@@ -43493,7 +43493,7 @@
       </c>
       <c r="C226" s="10" t="inlineStr">
         <is>
-          <t>SOES280 HYDROCLIMATE</t>
+          <t>SOES269 GIS FOR THE NATURAL ENVIRONMENT</t>
         </is>
       </c>
       <c r="D226" s="10" t="inlineStr">
@@ -43503,12 +43503,12 @@
       </c>
       <c r="E226" s="10" t="inlineStr">
         <is>
-          <t>SOE280 How the Earth's Climate System Works (3 credits)</t>
+          <t>SOE 486 Applied Remote Sensing: From Drones to Satellites</t>
         </is>
       </c>
       <c r="F226" s="10" t="inlineStr">
         <is>
-          <t>Level 2</t>
+          <t>Upper-level undergraduate</t>
         </is>
       </c>
       <c r="G226" s="10" t="inlineStr">
@@ -43518,18 +43518,18 @@
       </c>
       <c r="H226" s="10" t="inlineStr">
         <is>
-          <t>Term not stated in catalogue</t>
+          <t>2026/27 course verified; exact section term not publicly retrieved</t>
         </is>
       </c>
       <c r="I226" s="10" t="n"/>
       <c r="J226" s="10" t="inlineStr">
         <is>
-          <t>Host: https://catalog.wsu.edu/Pullman/Academics/Courses/SOE | NEW (Jul 2025 handbook, not previously in this file) - verified in current host catalogue, Oct 2026 via web search | UoL match is a SUGGESTION for department review (programme LOs, not close module match)</t>
+          <t>Host: https://environment.wsu.edu/undergraduate-studies/bs-in-earth-and-environmental-sciences/earth-science/ | UoL: https://www.liverpool.ac.uk/courses/geography-bsc-hons</t>
         </is>
       </c>
       <c r="K226" s="10" t="inlineStr">
         <is>
-          <t>Added Oct 2026: July 2025 handbook module verified in current catalogue; UoL match is a suggestion for review; NOT OFFERED 2026/27: Not in Fall 2026 Pullman schedule [https://schedules.wsu.edu/ (Schedule of Classes, Fall 2026, Pullman)]</t>
+          <t>Original row; NOT OFFERED 2026/27: Not in Fall 2026 Pullman schedule [https://schedules.wsu.edu/ (Schedule of Classes, Fall 2026, Pullman)]</t>
         </is>
       </c>
     </row>
@@ -43546,7 +43546,7 @@
       </c>
       <c r="C227" s="10" t="inlineStr">
         <is>
-          <t>SOES269 GIS FOR THE NATURAL ENVIRONMENT</t>
+          <t>SOES280 HYDROCLIMATE</t>
         </is>
       </c>
       <c r="D227" s="10" t="inlineStr">
@@ -43556,12 +43556,12 @@
       </c>
       <c r="E227" s="10" t="inlineStr">
         <is>
-          <t>SOIL SCI 374 Remote Sensing &amp; Airphoto Interpretation</t>
+          <t>SOE280 How the Earth's Climate System Works (3 credits)</t>
         </is>
       </c>
       <c r="F227" s="10" t="inlineStr">
         <is>
-          <t>Level 3</t>
+          <t>Level 2</t>
         </is>
       </c>
       <c r="G227" s="10" t="inlineStr">
@@ -43571,18 +43571,18 @@
       </c>
       <c r="H227" s="10" t="inlineStr">
         <is>
-          <t>2026/27 course verified; exact section term not publicly retrieved</t>
+          <t>Term not stated in catalogue</t>
         </is>
       </c>
       <c r="I227" s="10" t="n"/>
       <c r="J227" s="10" t="inlineStr">
         <is>
-          <t>Host: https://environment.wsu.edu/undergraduate-studies/bs-in-earth-and-environmental-sciences/earth-science/ | UoL: https://www.liverpool.ac.uk/courses/geography-bsc-hons</t>
+          <t>Host: https://catalog.wsu.edu/Pullman/Academics/Courses/SOE | NEW (Jul 2025 handbook, not previously in this file) - verified in current host catalogue, Oct 2026 via web search | UoL match is a SUGGESTION for department review (programme LOs, not close module match)</t>
         </is>
       </c>
       <c r="K227" s="10" t="inlineStr">
         <is>
-          <t>Original row; NOT OFFERED 2026/27: Not in Fall 2026 Pullman schedule [https://schedules.wsu.edu/ (Schedule of Classes, Fall 2026, Pullman)]</t>
+          <t>Added Oct 2026: July 2025 handbook module verified in current catalogue; UoL match is a suggestion for review; NOT OFFERED 2026/27: Not in Fall 2026 Pullman schedule [https://schedules.wsu.edu/ (Schedule of Classes, Fall 2026, Pullman)]</t>
         </is>
       </c>
     </row>
@@ -43609,12 +43609,12 @@
       </c>
       <c r="E228" s="10" t="inlineStr">
         <is>
-          <t>SOIL SCI 468 GIS Spatial Analysis</t>
+          <t>SOIL SCI 374 Remote Sensing &amp; Airphoto Interpretation</t>
         </is>
       </c>
       <c r="F228" s="10" t="inlineStr">
         <is>
-          <t>Upper-level undergraduate</t>
+          <t>Level 3</t>
         </is>
       </c>
       <c r="G228" s="10" t="inlineStr">
@@ -43642,17 +43642,17 @@
     <row r="229">
       <c r="A229" s="10" t="inlineStr">
         <is>
-          <t>Western University — Canada</t>
+          <t>Washington State University — USA</t>
         </is>
       </c>
       <c r="B229" s="10" t="inlineStr">
         <is>
-          <t>Geography BA</t>
+          <t>Geography BSc</t>
         </is>
       </c>
       <c r="C229" s="10" t="inlineStr">
         <is>
-          <t>SOES270 RETHINKING NATURE: ENVIRONMENTAL KNOWLEDGE, SCIENCE AND SOCIETY</t>
+          <t>SOES269 GIS FOR THE NATURAL ENVIRONMENT</t>
         </is>
       </c>
       <c r="D229" s="10" t="inlineStr">
@@ -43662,12 +43662,12 @@
       </c>
       <c r="E229" s="10" t="inlineStr">
         <is>
-          <t>GEOGENV1400G Introduction to the Human Environment (0.5)</t>
+          <t>SOIL SCI 468 GIS Spatial Analysis</t>
         </is>
       </c>
       <c r="F229" s="10" t="inlineStr">
         <is>
-          <t>Level 1</t>
+          <t>Upper-level undergraduate</t>
         </is>
       </c>
       <c r="G229" s="10" t="inlineStr">
@@ -43677,18 +43677,18 @@
       </c>
       <c r="H229" s="10" t="inlineStr">
         <is>
-          <t>2026/27 course verified; exact section term not publicly retrievable</t>
+          <t>2026/27 course verified; exact section term not publicly retrieved</t>
         </is>
       </c>
       <c r="I229" s="10" t="n"/>
       <c r="J229" s="10" t="inlineStr">
         <is>
-          <t>Host: https://geoenvironment.uwo.ca/ | UoL: https://www.liverpool.ac.uk/courses/geography-ba-hons</t>
+          <t>Host: https://environment.wsu.edu/undergraduate-studies/bs-in-earth-and-environmental-sciences/earth-science/ | UoL: https://www.liverpool.ac.uk/courses/geography-bsc-hons</t>
         </is>
       </c>
       <c r="K229" s="10" t="inlineStr">
         <is>
-          <t>Original row; WRONG TERM 2026/27: Winter 2027 only (suffix G) [https://studentservices.uwo.ca/secure/timetables/mastertt/ttindex.cfm]</t>
+          <t>Original row; NOT OFFERED 2026/27: Not in Fall 2026 Pullman schedule [https://schedules.wsu.edu/ (Schedule of Classes, Fall 2026, Pullman)]</t>
         </is>
       </c>
     </row>
@@ -43705,7 +43705,7 @@
       </c>
       <c r="C230" s="10" t="inlineStr">
         <is>
-          <t>SOES225 THEMES IN URBAN GEOGRAPHY</t>
+          <t>SOES270 RETHINKING NATURE: ENVIRONMENTAL KNOWLEDGE, SCIENCE AND SOCIETY</t>
         </is>
       </c>
       <c r="D230" s="10" t="inlineStr">
@@ -43715,12 +43715,12 @@
       </c>
       <c r="E230" s="10" t="inlineStr">
         <is>
-          <t>GEOGENV2460F/G Introduction to Urban Development</t>
+          <t>GEOGENV1400G Introduction to the Human Environment (0.5)</t>
         </is>
       </c>
       <c r="F230" s="10" t="inlineStr">
         <is>
-          <t>Level 2</t>
+          <t>Level 1</t>
         </is>
       </c>
       <c r="G230" s="10" t="inlineStr">
@@ -43768,12 +43768,12 @@
       </c>
       <c r="E231" s="10" t="inlineStr">
         <is>
-          <t>GEOGENV3354A/B Water And Cities (0.5 course)</t>
+          <t>GEOGENV2460F/G Introduction to Urban Development</t>
         </is>
       </c>
       <c r="F231" s="10" t="inlineStr">
         <is>
-          <t>Level 3</t>
+          <t>Level 2</t>
         </is>
       </c>
       <c r="G231" s="10" t="inlineStr">
@@ -43783,18 +43783,18 @@
       </c>
       <c r="H231" s="10" t="inlineStr">
         <is>
-          <t>Suffix 3354A/B (A=Fall, B=Winter)</t>
+          <t>2026/27 course verified; exact section term not publicly retrievable</t>
         </is>
       </c>
       <c r="I231" s="10" t="n"/>
       <c r="J231" s="10" t="inlineStr">
         <is>
-          <t>Host: https://www.westerncalendar.uwo.ca/Courses.cfm?SelectedCalendar=Live&amp;ArchiveID=&amp;Subject=GEOGENV | NEW (Jul 2025 handbook, not previously in this file) - verified in current host catalogue, Oct 2026 | UoL match is a SUGGESTION for department review (programme LOs, not close module match)</t>
+          <t>Host: https://geoenvironment.uwo.ca/ | UoL: https://www.liverpool.ac.uk/courses/geography-ba-hons</t>
         </is>
       </c>
       <c r="K231" s="10" t="inlineStr">
         <is>
-          <t>Added Oct 2026: July 2025 handbook module verified in current catalogue; UoL match is a suggestion for review; NOT OFFERED 2026/27: Not in the 2026/27 timetable [https://studentservices.uwo.ca/secure/timetables/mastertt/ttindex.cfm]</t>
+          <t>Original row; WRONG TERM 2026/27: Winter 2027 only (suffix G) [https://studentservices.uwo.ca/secure/timetables/mastertt/ttindex.cfm]</t>
         </is>
       </c>
     </row>
@@ -43806,12 +43806,12 @@
       </c>
       <c r="B232" s="10" t="inlineStr">
         <is>
-          <t>Geography BSc</t>
+          <t>Geography BA</t>
         </is>
       </c>
       <c r="C232" s="10" t="inlineStr">
         <is>
-          <t>SOES214 CHANGING ENVIRONMENTS</t>
+          <t>SOES225 THEMES IN URBAN GEOGRAPHY</t>
         </is>
       </c>
       <c r="D232" s="10" t="inlineStr">
@@ -43821,12 +43821,12 @@
       </c>
       <c r="E232" s="10" t="inlineStr">
         <is>
-          <t>GEOGENV1300A/B Introduction to the Physical Environment (0.5)</t>
+          <t>GEOGENV3354A/B Water And Cities (0.5 course)</t>
         </is>
       </c>
       <c r="F232" s="10" t="inlineStr">
         <is>
-          <t>Level 1</t>
+          <t>Level 3</t>
         </is>
       </c>
       <c r="G232" s="10" t="inlineStr">
@@ -43836,18 +43836,18 @@
       </c>
       <c r="H232" s="10" t="inlineStr">
         <is>
-          <t>2026/27 course verified; exact section term not publicly retrievable</t>
+          <t>Suffix 3354A/B (A=Fall, B=Winter)</t>
         </is>
       </c>
       <c r="I232" s="10" t="n"/>
       <c r="J232" s="10" t="inlineStr">
         <is>
-          <t>Host: https://geoenvironment.uwo.ca/ | UoL: https://www.liverpool.ac.uk/courses/geography-bsc-hons</t>
+          <t>Host: https://www.westerncalendar.uwo.ca/Courses.cfm?SelectedCalendar=Live&amp;ArchiveID=&amp;Subject=GEOGENV | NEW (Jul 2025 handbook, not previously in this file) - verified in current host catalogue, Oct 2026 | UoL match is a SUGGESTION for department review (programme LOs, not close module match)</t>
         </is>
       </c>
       <c r="K232" s="10" t="inlineStr">
         <is>
-          <t>Original row; WRONG TERM 2026/27: Winter 2027 only (suffix B) [https://studentservices.uwo.ca/secure/timetables/mastertt/ttindex.cfm]</t>
+          <t>Added Oct 2026: July 2025 handbook module verified in current catalogue; UoL match is a suggestion for review; NOT OFFERED 2026/27: Not in the 2026/27 timetable [https://studentservices.uwo.ca/secure/timetables/mastertt/ttindex.cfm]</t>
         </is>
       </c>
     </row>
@@ -43874,12 +43874,12 @@
       </c>
       <c r="E233" s="10" t="inlineStr">
         <is>
-          <t>GEOGENV2131A/B Natural Environment</t>
+          <t>GEOGENV1300A/B Introduction to the Physical Environment (0.5)</t>
         </is>
       </c>
       <c r="F233" s="10" t="inlineStr">
         <is>
-          <t>Level 2</t>
+          <t>Level 1</t>
         </is>
       </c>
       <c r="G233" s="10" t="inlineStr">
@@ -43900,7 +43900,7 @@
       </c>
       <c r="K233" s="10" t="inlineStr">
         <is>
-          <t>Original row; NOT OFFERED 2026/27: Not in the 2026/27 timetable [https://studentservices.uwo.ca/secure/timetables/mastertt/ttindex.cfm]</t>
+          <t>Original row; WRONG TERM 2026/27: Winter 2027 only (suffix B) [https://studentservices.uwo.ca/secure/timetables/mastertt/ttindex.cfm]</t>
         </is>
       </c>
     </row>
@@ -43917,7 +43917,7 @@
       </c>
       <c r="C234" s="10" t="inlineStr">
         <is>
-          <t>SOES269 GIS FOR THE NATURAL ENVIRONMENT</t>
+          <t>SOES214 CHANGING ENVIRONMENTS</t>
         </is>
       </c>
       <c r="D234" s="10" t="inlineStr">
@@ -43927,7 +43927,7 @@
       </c>
       <c r="E234" s="10" t="inlineStr">
         <is>
-          <t>GEOGENV2230A/B Remote Sensing</t>
+          <t>GEOGENV2131A/B Natural Environment</t>
         </is>
       </c>
       <c r="F234" s="10" t="inlineStr">
@@ -43953,7 +43953,7 @@
       </c>
       <c r="K234" s="10" t="inlineStr">
         <is>
-          <t>Original row; WRONG TERM 2026/27: Winter 2027 only (suffix B) [https://studentservices.uwo.ca/secure/timetables/mastertt/ttindex.cfm]</t>
+          <t>Original row; NOT OFFERED 2026/27: Not in the 2026/27 timetable [https://studentservices.uwo.ca/secure/timetables/mastertt/ttindex.cfm]</t>
         </is>
       </c>
     </row>
@@ -43970,7 +43970,7 @@
       </c>
       <c r="C235" s="10" t="inlineStr">
         <is>
-          <t>SOES280 HYDROCLIMATE</t>
+          <t>SOES269 GIS FOR THE NATURAL ENVIRONMENT</t>
         </is>
       </c>
       <c r="D235" s="10" t="inlineStr">
@@ -43980,7 +43980,7 @@
       </c>
       <c r="E235" s="10" t="inlineStr">
         <is>
-          <t>GEOGENV2330A/B Geomorphology and Hydrology</t>
+          <t>GEOGENV2230A/B Remote Sensing</t>
         </is>
       </c>
       <c r="F235" s="10" t="inlineStr">
@@ -44006,7 +44006,7 @@
       </c>
       <c r="K235" s="10" t="inlineStr">
         <is>
-          <t>Original row; NOT OFFERED 2026/27: Not in the 2026/27 timetable [https://studentservices.uwo.ca/secure/timetables/mastertt/ttindex.cfm]</t>
+          <t>Original row; WRONG TERM 2026/27: Winter 2027 only (suffix B) [https://studentservices.uwo.ca/secure/timetables/mastertt/ttindex.cfm]</t>
         </is>
       </c>
     </row>
@@ -44023,7 +44023,7 @@
       </c>
       <c r="C236" s="10" t="inlineStr">
         <is>
-          <t>SOES269 GIS FOR THE NATURAL ENVIRONMENT</t>
+          <t>SOES280 HYDROCLIMATE</t>
         </is>
       </c>
       <c r="D236" s="10" t="inlineStr">
@@ -44033,12 +44033,12 @@
       </c>
       <c r="E236" s="10" t="inlineStr">
         <is>
-          <t>GEOGENV3222A/B Geographic Information Science II</t>
+          <t>GEOGENV2330A/B Geomorphology and Hydrology</t>
         </is>
       </c>
       <c r="F236" s="10" t="inlineStr">
         <is>
-          <t>Level 3</t>
+          <t>Level 2</t>
         </is>
       </c>
       <c r="G236" s="10" t="inlineStr">
@@ -44059,7 +44059,7 @@
       </c>
       <c r="K236" s="10" t="inlineStr">
         <is>
-          <t>Original row; WRONG TERM 2026/27: Winter 2027 only (suffix B) [https://studentservices.uwo.ca/secure/timetables/mastertt/ttindex.cfm]</t>
+          <t>Original row; NOT OFFERED 2026/27: Not in the 2026/27 timetable [https://studentservices.uwo.ca/secure/timetables/mastertt/ttindex.cfm]</t>
         </is>
       </c>
     </row>
@@ -44076,7 +44076,7 @@
       </c>
       <c r="C237" s="10" t="inlineStr">
         <is>
-          <t>SOES280 HYDROCLIMATE</t>
+          <t>SOES269 GIS FOR THE NATURAL ENVIRONMENT</t>
         </is>
       </c>
       <c r="D237" s="10" t="inlineStr">
@@ -44086,7 +44086,7 @@
       </c>
       <c r="E237" s="10" t="inlineStr">
         <is>
-          <t>GEOGENV3354A/B Water And Cities (0.5 course)</t>
+          <t>GEOGENV3222A/B Geographic Information Science II</t>
         </is>
       </c>
       <c r="F237" s="10" t="inlineStr">
@@ -44101,18 +44101,18 @@
       </c>
       <c r="H237" s="10" t="inlineStr">
         <is>
-          <t>Suffix 3354A/B (A=Fall, B=Winter)</t>
+          <t>2026/27 course verified; exact section term not publicly retrievable</t>
         </is>
       </c>
       <c r="I237" s="10" t="n"/>
       <c r="J237" s="10" t="inlineStr">
         <is>
-          <t>Host: https://www.westerncalendar.uwo.ca/Courses.cfm?SelectedCalendar=Live&amp;ArchiveID=&amp;Subject=GEOGENV | NEW (Jul 2025 handbook, not previously in this file) - verified in current host catalogue, Oct 2026 | UoL match is a SUGGESTION for department review (programme LOs, not close module match)</t>
+          <t>Host: https://geoenvironment.uwo.ca/ | UoL: https://www.liverpool.ac.uk/courses/geography-bsc-hons</t>
         </is>
       </c>
       <c r="K237" s="10" t="inlineStr">
         <is>
-          <t>Added Oct 2026: July 2025 handbook module verified in current catalogue; UoL match is a suggestion for review; NOT OFFERED 2026/27: Not in the 2026/27 timetable [https://studentservices.uwo.ca/secure/timetables/mastertt/ttindex.cfm]</t>
+          <t>Original row; WRONG TERM 2026/27: Winter 2027 only (suffix B) [https://studentservices.uwo.ca/secure/timetables/mastertt/ttindex.cfm]</t>
         </is>
       </c>
     </row>
@@ -44129,7 +44129,7 @@
       </c>
       <c r="C238" s="10" t="inlineStr">
         <is>
-          <t>SOES269 GIS FOR THE NATURAL ENVIRONMENT</t>
+          <t>SOES280 HYDROCLIMATE</t>
         </is>
       </c>
       <c r="D238" s="10" t="inlineStr">
@@ -44139,12 +44139,12 @@
       </c>
       <c r="E238" s="10" t="inlineStr">
         <is>
-          <t>GEOGENV4230A/B Advanced Topics in Remote Sensing</t>
+          <t>GEOGENV3354A/B Water And Cities (0.5 course)</t>
         </is>
       </c>
       <c r="F238" s="10" t="inlineStr">
         <is>
-          <t>Upper-level undergraduate</t>
+          <t>Level 3</t>
         </is>
       </c>
       <c r="G238" s="10" t="inlineStr">
@@ -44154,35 +44154,35 @@
       </c>
       <c r="H238" s="10" t="inlineStr">
         <is>
-          <t>2026/27 course verified; exact section term not publicly retrievable</t>
+          <t>Suffix 3354A/B (A=Fall, B=Winter)</t>
         </is>
       </c>
       <c r="I238" s="10" t="n"/>
       <c r="J238" s="10" t="inlineStr">
         <is>
-          <t>Host: https://geoenvironment.uwo.ca/ | UoL: https://www.liverpool.ac.uk/courses/geography-bsc-hons</t>
+          <t>Host: https://www.westerncalendar.uwo.ca/Courses.cfm?SelectedCalendar=Live&amp;ArchiveID=&amp;Subject=GEOGENV | NEW (Jul 2025 handbook, not previously in this file) - verified in current host catalogue, Oct 2026 | UoL match is a SUGGESTION for department review (programme LOs, not close module match)</t>
         </is>
       </c>
       <c r="K238" s="10" t="inlineStr">
         <is>
-          <t>Original row; WRONG TERM 2026/27: Winter 2027 only (suffix B) [https://studentservices.uwo.ca/secure/timetables/mastertt/ttindex.cfm]</t>
+          <t>Added Oct 2026: July 2025 handbook module verified in current catalogue; UoL match is a suggestion for review; NOT OFFERED 2026/27: Not in the 2026/27 timetable [https://studentservices.uwo.ca/secure/timetables/mastertt/ttindex.cfm]</t>
         </is>
       </c>
     </row>
     <row r="239">
       <c r="A239" s="10" t="inlineStr">
         <is>
-          <t>Western Washington University — USA</t>
+          <t>Western University — Canada</t>
         </is>
       </c>
       <c r="B239" s="10" t="inlineStr">
         <is>
-          <t>Geography BA</t>
+          <t>Geography BSc</t>
         </is>
       </c>
       <c r="C239" s="10" t="inlineStr">
         <is>
-          <t>SOES270 RETHINKING NATURE: ENVIRONMENTAL KNOWLEDGE, SCIENCE AND SOCIETY</t>
+          <t>SOES269 GIS FOR THE NATURAL ENVIRONMENT</t>
         </is>
       </c>
       <c r="D239" s="10" t="inlineStr">
@@ -44192,12 +44192,12 @@
       </c>
       <c r="E239" s="10" t="inlineStr">
         <is>
-          <t>ENVS 204 Human Geography (4 credits)</t>
+          <t>GEOGENV4230A/B Advanced Topics in Remote Sensing</t>
         </is>
       </c>
       <c r="F239" s="10" t="inlineStr">
         <is>
-          <t>Level 2</t>
+          <t>Upper-level undergraduate</t>
         </is>
       </c>
       <c r="G239" s="10" t="inlineStr">
@@ -44207,18 +44207,18 @@
       </c>
       <c r="H239" s="10" t="inlineStr">
         <is>
-          <t>Winter</t>
+          <t>2026/27 course verified; exact section term not publicly retrievable</t>
         </is>
       </c>
       <c r="I239" s="10" t="n"/>
       <c r="J239" s="10" t="inlineStr">
         <is>
-          <t>Host: https://cenv.wwu.edu/FAQs-ENVS-declared-students | UoL: https://www.liverpool.ac.uk/courses/geography-ba-hons</t>
+          <t>Host: https://geoenvironment.uwo.ca/ | UoL: https://www.liverpool.ac.uk/courses/geography-bsc-hons</t>
         </is>
       </c>
       <c r="K239" s="10" t="inlineStr">
         <is>
-          <t>Original row; Wrong term for partner semester (Fall Semester [Sep-Dec))</t>
+          <t>Original row; WRONG TERM 2026/27: Winter 2027 only (suffix B) [https://studentservices.uwo.ca/secure/timetables/mastertt/ttindex.cfm]</t>
         </is>
       </c>
     </row>
@@ -44235,7 +44235,7 @@
       </c>
       <c r="C240" s="10" t="inlineStr">
         <is>
-          <t>SOES275 SOCIAL AND CULTURAL GEOGRAPHIES</t>
+          <t>SOES270 RETHINKING NATURE: ENVIRONMENTAL KNOWLEDGE, SCIENCE AND SOCIETY</t>
         </is>
       </c>
       <c r="D240" s="10" t="inlineStr">
@@ -44245,12 +44245,12 @@
       </c>
       <c r="E240" s="10" t="inlineStr">
         <is>
-          <t>ENVS 331 Canada: Society and Environment (4 credits)</t>
+          <t>ENVS 204 Human Geography (4 credits)</t>
         </is>
       </c>
       <c r="F240" s="10" t="inlineStr">
         <is>
-          <t>Level 3</t>
+          <t>Level 2</t>
         </is>
       </c>
       <c r="G240" s="10" t="inlineStr">
@@ -44260,7 +44260,7 @@
       </c>
       <c r="H240" s="10" t="inlineStr">
         <is>
-          <t>2026/27 catalogue verified; exact quarter not publicly specified</t>
+          <t>Winter</t>
         </is>
       </c>
       <c r="I240" s="10" t="n"/>
@@ -44271,7 +44271,7 @@
       </c>
       <c r="K240" s="10" t="inlineStr">
         <is>
-          <t>Original row; NOT OFFERED 2026/27: Not in Fall 2026 quarter [https://registration.banner.wwu.edu/StudentRegistrationSsb/ssb/term/termSelection?mode=search (Browse Classes, Fall 2026 quarter)]</t>
+          <t>Original row; Wrong term for partner semester (Fall Semester [Sep-Dec))</t>
         </is>
       </c>
     </row>
@@ -44288,7 +44288,7 @@
       </c>
       <c r="C241" s="10" t="inlineStr">
         <is>
-          <t>SOES270 RETHINKING NATURE: ENVIRONMENTAL KNOWLEDGE, SCIENCE AND SOCIETY</t>
+          <t>SOES275 SOCIAL AND CULTURAL GEOGRAPHIES</t>
         </is>
       </c>
       <c r="D241" s="10" t="inlineStr">
@@ -44298,7 +44298,7 @@
       </c>
       <c r="E241" s="10" t="inlineStr">
         <is>
-          <t>ENVS 340 Developing World</t>
+          <t>ENVS 331 Canada: Society and Environment (4 credits)</t>
         </is>
       </c>
       <c r="F241" s="10" t="inlineStr">
@@ -44351,7 +44351,7 @@
       </c>
       <c r="E242" s="10" t="inlineStr">
         <is>
-          <t>ENVS327 The Soil Environment</t>
+          <t>ENVS 340 Developing World</t>
         </is>
       </c>
       <c r="F242" s="10" t="inlineStr">
@@ -44366,18 +44366,18 @@
       </c>
       <c r="H242" s="10" t="inlineStr">
         <is>
-          <t>Term not stated in catalogue</t>
+          <t>2026/27 catalogue verified; exact quarter not publicly specified</t>
         </is>
       </c>
       <c r="I242" s="10" t="n"/>
       <c r="J242" s="10" t="inlineStr">
         <is>
-          <t>Host: https://catalog.wwu.edu/ | NEW (Jul 2025 handbook, not previously in this file) - verified in current host catalogue, Oct 2026 via web search | UoL match is a SUGGESTION for department review (programme LOs, not close module match)</t>
+          <t>Host: https://cenv.wwu.edu/FAQs-ENVS-declared-students | UoL: https://www.liverpool.ac.uk/courses/geography-ba-hons</t>
         </is>
       </c>
       <c r="K242" s="10" t="inlineStr">
         <is>
-          <t>Added Oct 2026: July 2025 handbook module verified in current catalogue; UoL match is a suggestion for review; NOT OFFERED 2026/27: Not in Fall 2026 quarter [https://registration.banner.wwu.edu/StudentRegistrationSsb/ssb/term/termSelection?mode=search (Browse Classes, Fall 2026 quarter)]</t>
+          <t>Original row; NOT OFFERED 2026/27: Not in Fall 2026 quarter [https://registration.banner.wwu.edu/StudentRegistrationSsb/ssb/term/termSelection?mode=search (Browse Classes, Fall 2026 quarter)]</t>
         </is>
       </c>
     </row>
@@ -44394,7 +44394,7 @@
       </c>
       <c r="C243" s="10" t="inlineStr">
         <is>
-          <t>SOES222 PLANNING FOR SUSTAINABLE URBANISM</t>
+          <t>SOES270 RETHINKING NATURE: ENVIRONMENTAL KNOWLEDGE, SCIENCE AND SOCIETY</t>
         </is>
       </c>
       <c r="D243" s="10" t="inlineStr">
@@ -44404,7 +44404,7 @@
       </c>
       <c r="E243" s="10" t="inlineStr">
         <is>
-          <t>ENVS372 Natural Hazards Planning</t>
+          <t>ENVS327 The Soil Environment</t>
         </is>
       </c>
       <c r="F243" s="10" t="inlineStr">
@@ -44447,7 +44447,7 @@
       </c>
       <c r="C244" s="10" t="inlineStr">
         <is>
-          <t>SOES270 RETHINKING NATURE: ENVIRONMENTAL KNOWLEDGE, SCIENCE AND SOCIETY</t>
+          <t>SOES222 PLANNING FOR SUSTAINABLE URBANISM</t>
         </is>
       </c>
       <c r="D244" s="10" t="inlineStr">
@@ -44457,7 +44457,7 @@
       </c>
       <c r="E244" s="10" t="inlineStr">
         <is>
-          <t>SOC 374 Sociology of Environmental Inequality and Justice</t>
+          <t>ENVS372 Natural Hazards Planning</t>
         </is>
       </c>
       <c r="F244" s="10" t="inlineStr">
@@ -44495,12 +44495,12 @@
       </c>
       <c r="B245" s="10" t="inlineStr">
         <is>
-          <t>Geography BSc</t>
+          <t>Geography BA</t>
         </is>
       </c>
       <c r="C245" s="10" t="inlineStr">
         <is>
-          <t>SOES218 GEOMORPHOLOGY: PROCESSES AND FORMS</t>
+          <t>SOES270 RETHINKING NATURE: ENVIRONMENTAL KNOWLEDGE, SCIENCE AND SOCIETY</t>
         </is>
       </c>
       <c r="D245" s="10" t="inlineStr">
@@ -44510,7 +44510,7 @@
       </c>
       <c r="E245" s="10" t="inlineStr">
         <is>
-          <t>ENVS325 Geography of Landforms</t>
+          <t>SOC 374 Sociology of Environmental Inequality and Justice</t>
         </is>
       </c>
       <c r="F245" s="10" t="inlineStr">
@@ -44563,7 +44563,7 @@
       </c>
       <c r="E246" s="10" t="inlineStr">
         <is>
-          <t>ENVS327 The Soil Environment</t>
+          <t>ENVS325 Geography of Landforms</t>
         </is>
       </c>
       <c r="F246" s="10" t="inlineStr">
@@ -44606,7 +44606,7 @@
       </c>
       <c r="C247" s="10" t="inlineStr">
         <is>
-          <t>SOES280 HYDROCLIMATE</t>
+          <t>SOES218 GEOMORPHOLOGY: PROCESSES AND FORMS</t>
         </is>
       </c>
       <c r="D247" s="10" t="inlineStr">
@@ -44616,7 +44616,7 @@
       </c>
       <c r="E247" s="10" t="inlineStr">
         <is>
-          <t>ENVS344 Community Solutions to Climate Change (4 credits)</t>
+          <t>ENVS327 The Soil Environment</t>
         </is>
       </c>
       <c r="F247" s="10" t="inlineStr">
@@ -44659,7 +44659,7 @@
       </c>
       <c r="C248" s="10" t="inlineStr">
         <is>
-          <t>SOES214 CHANGING ENVIRONMENTS</t>
+          <t>SOES280 HYDROCLIMATE</t>
         </is>
       </c>
       <c r="D248" s="10" t="inlineStr">
@@ -44669,7 +44669,7 @@
       </c>
       <c r="E248" s="10" t="inlineStr">
         <is>
-          <t>ENVS372 Natural Hazards Planning</t>
+          <t>ENVS344 Community Solutions to Climate Change (4 credits)</t>
         </is>
       </c>
       <c r="F248" s="10" t="inlineStr">
@@ -44712,7 +44712,7 @@
       </c>
       <c r="C249" s="10" t="inlineStr">
         <is>
-          <t>SOES269 GIS FOR THE NATURAL ENVIRONMENT</t>
+          <t>SOES214 CHANGING ENVIRONMENTS</t>
         </is>
       </c>
       <c r="D249" s="10" t="inlineStr">
@@ -44722,12 +44722,12 @@
       </c>
       <c r="E249" s="10" t="inlineStr">
         <is>
-          <t>ENVS419 Applications in GIS</t>
+          <t>ENVS372 Natural Hazards Planning</t>
         </is>
       </c>
       <c r="F249" s="10" t="inlineStr">
         <is>
-          <t>Upper-level undergraduate</t>
+          <t>Level 3</t>
         </is>
       </c>
       <c r="G249" s="10" t="inlineStr">
@@ -44737,18 +44737,18 @@
       </c>
       <c r="H249" s="10" t="inlineStr">
         <is>
-          <t>2026/27 catalogue verified; exact quarter not publicly specified</t>
+          <t>Term not stated in catalogue</t>
         </is>
       </c>
       <c r="I249" s="10" t="n"/>
       <c r="J249" s="10" t="inlineStr">
         <is>
-          <t>Host: https://cenv.wwu.edu/FAQs-ENVS-declared-students | UoL: https://www.liverpool.ac.uk/courses/geography-bsc-hons</t>
+          <t>Host: https://catalog.wwu.edu/ | NEW (Jul 2025 handbook, not previously in this file) - verified in current host catalogue, Oct 2026 via web search | UoL match is a SUGGESTION for department review (programme LOs, not close module match)</t>
         </is>
       </c>
       <c r="K249" s="10" t="inlineStr">
         <is>
-          <t>Original row; NOT OFFERED 2026/27: Not in Fall 2026 quarter [https://registration.banner.wwu.edu/StudentRegistrationSsb/ssb/term/termSelection?mode=search (Browse Classes, Fall 2026 quarter)]</t>
+          <t>Added Oct 2026: July 2025 handbook module verified in current catalogue; UoL match is a suggestion for review; NOT OFFERED 2026/27: Not in Fall 2026 quarter [https://registration.banner.wwu.edu/StudentRegistrationSsb/ssb/term/termSelection?mode=search (Browse Classes, Fall 2026 quarter)]</t>
         </is>
       </c>
     </row>
@@ -44775,7 +44775,7 @@
       </c>
       <c r="E250" s="10" t="inlineStr">
         <is>
-          <t>ENVS421 GIS IV: Geospatial Data Creation and Management</t>
+          <t>ENVS419 Applications in GIS</t>
         </is>
       </c>
       <c r="F250" s="10" t="inlineStr">
@@ -44828,7 +44828,7 @@
       </c>
       <c r="E251" s="10" t="inlineStr">
         <is>
-          <t>ESCI442 Introduction to Remote Sensing</t>
+          <t>ENVS421 GIS IV: Geospatial Data Creation and Management</t>
         </is>
       </c>
       <c r="F251" s="10" t="inlineStr">
@@ -44858,8 +44858,61 @@
         </is>
       </c>
     </row>
+    <row r="252">
+      <c r="A252" s="10" t="inlineStr">
+        <is>
+          <t>Western Washington University — USA</t>
+        </is>
+      </c>
+      <c r="B252" s="10" t="inlineStr">
+        <is>
+          <t>Geography BSc</t>
+        </is>
+      </c>
+      <c r="C252" s="10" t="inlineStr">
+        <is>
+          <t>SOES269 GIS FOR THE NATURAL ENVIRONMENT</t>
+        </is>
+      </c>
+      <c r="D252" s="10" t="inlineStr">
+        <is>
+          <t>Level 5</t>
+        </is>
+      </c>
+      <c r="E252" s="10" t="inlineStr">
+        <is>
+          <t>ESCI442 Introduction to Remote Sensing</t>
+        </is>
+      </c>
+      <c r="F252" s="10" t="inlineStr">
+        <is>
+          <t>Upper-level undergraduate</t>
+        </is>
+      </c>
+      <c r="G252" s="10" t="inlineStr">
+        <is>
+          <t>Optional</t>
+        </is>
+      </c>
+      <c r="H252" s="10" t="inlineStr">
+        <is>
+          <t>2026/27 catalogue verified; exact quarter not publicly specified</t>
+        </is>
+      </c>
+      <c r="I252" s="10" t="n"/>
+      <c r="J252" s="10" t="inlineStr">
+        <is>
+          <t>Host: https://cenv.wwu.edu/FAQs-ENVS-declared-students | UoL: https://www.liverpool.ac.uk/courses/geography-bsc-hons</t>
+        </is>
+      </c>
+      <c r="K252" s="10" t="inlineStr">
+        <is>
+          <t>Original row; NOT OFFERED 2026/27: Not in Fall 2026 quarter [https://registration.banner.wwu.edu/StudentRegistrationSsb/ssb/term/termSelection?mode=search (Browse Classes, Fall 2026 quarter)]</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:K251"/>
+  <autoFilter ref="A1:K252"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Kansas State BA: typical offering terms
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01EZa6h9SpqLeB7ZbHz6KiwN
</commit_message>
<xml_diff>
--- a/curriculum_mapping_2026-27/CurriculumMapping_Geo_1_ReviewEntry_OK.xlsx
+++ b/curriculum_mapping_2026-27/CurriculumMapping_Geo_1_ReviewEntry_OK.xlsx
@@ -1065,17 +1065,17 @@
         </is>
       </c>
       <c r="C18" s="3" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="D18" s="3" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="E18" s="3" t="n">
         <v>4</v>
       </c>
       <c r="F18" s="4" t="inlineStr">
         <is>
-          <t>Meets minimum, little choice: 4 modules with confirmed 2026/27 term, 4 needed (+5 more with unverified term)</t>
+          <t>OK: 7 modules with confirmed 2026/27 term, 4 needed (+2 more with unverified term)</t>
         </is>
       </c>
       <c r="G18" s="3" t="inlineStr">
@@ -6195,55 +6195,55 @@
       </c>
     </row>
     <row r="48">
-      <c r="A48" s="4" t="inlineStr">
+      <c r="A48" s="6" t="inlineStr">
         <is>
           <t>Kansas State University — USA</t>
         </is>
       </c>
-      <c r="B48" s="4" t="inlineStr">
+      <c r="B48" s="6" t="inlineStr">
         <is>
           <t>Geography BA</t>
         </is>
       </c>
-      <c r="C48" s="4" t="inlineStr">
+      <c r="C48" s="6" t="inlineStr">
         <is>
           <t>SOES224 POLITICAL ECONOMIES OF CRISIS AND CHANGE</t>
         </is>
       </c>
-      <c r="D48" s="4" t="inlineStr">
-        <is>
-          <t>Level 5</t>
-        </is>
-      </c>
-      <c r="E48" s="4" t="inlineStr">
+      <c r="D48" s="6" t="inlineStr">
+        <is>
+          <t>Level 5</t>
+        </is>
+      </c>
+      <c r="E48" s="6" t="inlineStr">
         <is>
           <t>GEOG100 World Geography &amp; Globalization (3 credits)</t>
         </is>
       </c>
-      <c r="F48" s="4" t="inlineStr">
+      <c r="F48" s="6" t="inlineStr">
         <is>
           <t>Level 1</t>
         </is>
       </c>
-      <c r="G48" s="4" t="inlineStr">
-        <is>
-          <t>Optional</t>
-        </is>
-      </c>
-      <c r="H48" s="4" t="inlineStr">
-        <is>
-          <t>Fall/Spring/Summer</t>
-        </is>
-      </c>
-      <c r="I48" s="4" t="n"/>
-      <c r="J48" s="4" t="inlineStr">
+      <c r="G48" s="6" t="inlineStr">
+        <is>
+          <t>Optional</t>
+        </is>
+      </c>
+      <c r="H48" s="6" t="inlineStr">
+        <is>
+          <t>Typically offered Fall, Spring, Summer</t>
+        </is>
+      </c>
+      <c r="I48" s="6" t="n"/>
+      <c r="J48" s="6" t="inlineStr">
         <is>
           <t>Host: https://catalog.k-state.edu/undergraduate/arts-sciences/geography-geospatial-sciences/ | UoL: https://www.liverpool.ac.uk/courses/geography-ba-hons</t>
         </is>
       </c>
-      <c r="K48" s="4" t="inlineStr">
-        <is>
-          <t>Original row; TERM NOT VERIFIED: Term not verifiable: K-State class schedule/catalogue bot-protected</t>
+      <c r="K48" s="6" t="inlineStr">
+        <is>
+          <t>Original row; TERM LIKELY (2026/27 timetable not yet published or pattern only): Typically offered Fall, Spring, Summer [https://catalog.k-state.edu/ (Course Typically Offered - checked manually Oct 2026)]</t>
         </is>
       </c>
     </row>
@@ -6402,60 +6402,60 @@
       </c>
       <c r="K51" s="4" t="inlineStr">
         <is>
-          <t>Added Oct 2026: July 2025 handbook module verified in current catalogue; UoL match is a suggestion for review; TERM NOT VERIFIED: Term not verifiable: K-State class schedule/catalogue bot-protected</t>
+          <t>Added Oct 2026: July 2025 handbook module verified in current catalogue; UoL match is a suggestion for review; TERM NOT VERIFIED: Typically offered: Other (irregular) — Irregular offering - check Fall 2026 schedule [https://catalog.k-state.edu/ (Course Typically Offered - checked manually Oct 2026)]</t>
         </is>
       </c>
     </row>
     <row r="52">
-      <c r="A52" s="4" t="inlineStr">
+      <c r="A52" s="6" t="inlineStr">
         <is>
           <t>Kansas State University — USA</t>
         </is>
       </c>
-      <c r="B52" s="4" t="inlineStr">
+      <c r="B52" s="6" t="inlineStr">
         <is>
           <t>Geography BA</t>
         </is>
       </c>
-      <c r="C52" s="4" t="inlineStr">
+      <c r="C52" s="6" t="inlineStr">
         <is>
           <t>SOES270 RETHINKING NATURE: ENVIRONMENTAL KNOWLEDGE, SCIENCE AND SOCIETY</t>
         </is>
       </c>
-      <c r="D52" s="4" t="inlineStr">
-        <is>
-          <t>Level 5</t>
-        </is>
-      </c>
-      <c r="E52" s="4" t="inlineStr">
+      <c r="D52" s="6" t="inlineStr">
+        <is>
+          <t>Level 5</t>
+        </is>
+      </c>
+      <c r="E52" s="6" t="inlineStr">
         <is>
           <t>GEOG340 Geography of Natural Resources (3 credits)</t>
         </is>
       </c>
-      <c r="F52" s="4" t="inlineStr">
+      <c r="F52" s="6" t="inlineStr">
         <is>
           <t>Level 3</t>
         </is>
       </c>
-      <c r="G52" s="4" t="inlineStr">
-        <is>
-          <t>Optional</t>
-        </is>
-      </c>
-      <c r="H52" s="4" t="inlineStr">
-        <is>
-          <t>2026/27 catalogue verified; exact offering term not publicly specified</t>
-        </is>
-      </c>
-      <c r="I52" s="4" t="n"/>
-      <c r="J52" s="4" t="inlineStr">
+      <c r="G52" s="6" t="inlineStr">
+        <is>
+          <t>Optional</t>
+        </is>
+      </c>
+      <c r="H52" s="6" t="inlineStr">
+        <is>
+          <t>Typically offered Fall</t>
+        </is>
+      </c>
+      <c r="I52" s="6" t="n"/>
+      <c r="J52" s="6" t="inlineStr">
         <is>
           <t>Host: https://catalog.k-state.edu/undergraduate/arts-sciences/geography-geospatial-sciences/ | UoL: https://www.liverpool.ac.uk/courses/geography-ba-hons</t>
         </is>
       </c>
-      <c r="K52" s="4" t="inlineStr">
-        <is>
-          <t>Original row; TERM NOT VERIFIED: Term not verifiable: K-State class schedule/catalogue bot-protected</t>
+      <c r="K52" s="6" t="inlineStr">
+        <is>
+          <t>Original row; TERM LIKELY (2026/27 timetable not yet published or pattern only): Typically offered Fall [https://catalog.k-state.edu/ (Course Typically Offered - checked manually Oct 2026)]</t>
         </is>
       </c>
     </row>
@@ -6513,55 +6513,55 @@
       </c>
     </row>
     <row r="54">
-      <c r="A54" s="4" t="inlineStr">
+      <c r="A54" s="6" t="inlineStr">
         <is>
           <t>Kansas State University — USA</t>
         </is>
       </c>
-      <c r="B54" s="4" t="inlineStr">
+      <c r="B54" s="6" t="inlineStr">
         <is>
           <t>Geography BA</t>
         </is>
       </c>
-      <c r="C54" s="4" t="inlineStr">
+      <c r="C54" s="6" t="inlineStr">
         <is>
           <t>SOES270 RETHINKING NATURE: ENVIRONMENTAL KNOWLEDGE, SCIENCE AND SOCIETY</t>
         </is>
       </c>
-      <c r="D54" s="4" t="inlineStr">
-        <is>
-          <t>Level 5</t>
-        </is>
-      </c>
-      <c r="E54" s="4" t="inlineStr">
+      <c r="D54" s="6" t="inlineStr">
+        <is>
+          <t>Level 5</t>
+        </is>
+      </c>
+      <c r="E54" s="6" t="inlineStr">
         <is>
           <t>GEOG370 Environmental Justice (3 credits)</t>
         </is>
       </c>
-      <c r="F54" s="4" t="inlineStr">
+      <c r="F54" s="6" t="inlineStr">
         <is>
           <t>Level 3</t>
         </is>
       </c>
-      <c r="G54" s="4" t="inlineStr">
-        <is>
-          <t>Optional</t>
-        </is>
-      </c>
-      <c r="H54" s="4" t="inlineStr">
-        <is>
-          <t>Term not stated in catalogue</t>
-        </is>
-      </c>
-      <c r="I54" s="4" t="n"/>
-      <c r="J54" s="4" t="inlineStr">
+      <c r="G54" s="6" t="inlineStr">
+        <is>
+          <t>Optional</t>
+        </is>
+      </c>
+      <c r="H54" s="6" t="inlineStr">
+        <is>
+          <t>Typically offered Fall, Spring</t>
+        </is>
+      </c>
+      <c r="I54" s="6" t="n"/>
+      <c r="J54" s="6" t="inlineStr">
         <is>
           <t>Host: https://catalog.k-state.edu/preview_course_nopop.php?catoid=62&amp;coid=431882 | NEW (Jul 2025 handbook, not previously in this file) - verified in current host catalogue, Oct 2026 via web search | UoL match is a SUGGESTION for department review (programme LOs, not close module match)</t>
         </is>
       </c>
-      <c r="K54" s="4" t="inlineStr">
-        <is>
-          <t>Added Oct 2026: July 2025 handbook module verified in current catalogue; UoL match is a suggestion for review; TERM NOT VERIFIED: Term not verifiable: K-State class schedule/catalogue bot-protected</t>
+      <c r="K54" s="6" t="inlineStr">
+        <is>
+          <t>Added Oct 2026: July 2025 handbook module verified in current catalogue; UoL match is a suggestion for review; TERM LIKELY (2026/27 timetable not yet published or pattern only): Typically offered Fall, Spring [https://catalog.k-state.edu/ (Course Typically Offered - checked manually Oct 2026)]</t>
         </is>
       </c>
     </row>
@@ -6614,7 +6614,7 @@
       </c>
       <c r="K55" s="4" t="inlineStr">
         <is>
-          <t>Added Oct 2026: July 2025 handbook module verified in current catalogue; UoL match is a suggestion for review; TERM NOT VERIFIED: Term not verifiable: K-State class schedule/catalogue bot-protected</t>
+          <t>Added Oct 2026: July 2025 handbook module verified in current catalogue; UoL match is a suggestion for review; TERM NOT VERIFIED: Typically offered Fall OR Spring (alternates) — Could be Spring only in 2026/27 - check Fall 2026 schedule [https://catalog.k-state.edu/ (Course Typically Offered - checked manually Oct 2026)]</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Show known offering info in Semester column for unconfirmed rows
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01EZa6h9SpqLeB7ZbHz6KiwN
</commit_message>
<xml_diff>
--- a/curriculum_mapping_2026-27/CurriculumMapping_Geo_1_ReviewEntry_OK.xlsx
+++ b/curriculum_mapping_2026-27/CurriculumMapping_Geo_1_ReviewEntry_OK.xlsx
@@ -7280,7 +7280,7 @@
       </c>
       <c r="H72" s="5" t="inlineStr">
         <is>
-          <t>Term not stated in catalogue</t>
+          <t>Typically offered: Other (irregular) - NOT CONFIRMED for this exchange period</t>
         </is>
       </c>
       <c r="I72" s="5" t="n"/>
@@ -7492,7 +7492,7 @@
       </c>
       <c r="H76" s="5" t="inlineStr">
         <is>
-          <t>Term not stated in catalogue</t>
+          <t>Typically offered Fall OR Spring (alternates) - NOT CONFIRMED for this exchange period</t>
         </is>
       </c>
       <c r="I76" s="5" t="n"/>

</xml_diff>